<commit_message>
v12.1: Match it 'Of Age' (age of consent) + 'Hard Line' (statutory child-rape penalties), Nigeria Muslim-majority (Pew 56%), top-bar All tab removed, values always on (show-values toggle removed), Google AdSense (ca-pub-5196178239625142) via RankdAds with ads.txt; 110 dailies to Jan 23 2027
</commit_message>
<xml_diff>
--- a/puzzles.xlsx
+++ b/puzzles.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'country_info'!$A$1:$L$222</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'hint_bank'!$A$1:$H$206</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'top5_puzzles'!$A$1:$O$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'match_puzzles'!$A$1:$P$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'match_puzzles'!$A$1:$Q$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6530,7 +6530,7 @@
         </is>
       </c>
       <c r="B103" s="3" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
@@ -8021,7 +8021,7 @@
         </is>
       </c>
       <c r="B130" s="3" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         </is>
       </c>
       <c r="B139" s="3" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
@@ -12868,7 +12868,7 @@
         </is>
       </c>
       <c r="B209" s="3" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
@@ -14798,7 +14798,7 @@
         </is>
       </c>
       <c r="B239" s="3" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
@@ -15109,7 +15109,7 @@
         </is>
       </c>
       <c r="B244" s="2" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
@@ -15800,7 +15800,7 @@
         </is>
       </c>
       <c r="B255" s="2" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
@@ -16746,7 +16746,7 @@
         </is>
       </c>
       <c r="B271" s="3" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
@@ -17041,7 +17041,7 @@
         </is>
       </c>
       <c r="B276" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
@@ -17340,7 +17340,7 @@
         </is>
       </c>
       <c r="B281" s="3" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
@@ -17639,7 +17639,7 @@
         </is>
       </c>
       <c r="B286" s="2" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
@@ -18330,7 +18330,7 @@
         </is>
       </c>
       <c r="B297" s="2" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
@@ -18629,7 +18629,7 @@
         </is>
       </c>
       <c r="B302" s="3" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
@@ -19272,7 +19272,7 @@
         </is>
       </c>
       <c r="B313" s="3" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
@@ -19567,7 +19567,7 @@
         </is>
       </c>
       <c r="B318" s="2" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
@@ -19866,7 +19866,7 @@
         </is>
       </c>
       <c r="B323" s="3" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
@@ -20165,7 +20165,7 @@
         </is>
       </c>
       <c r="B328" s="2" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
@@ -20464,7 +20464,7 @@
         </is>
       </c>
       <c r="B333" s="3" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
@@ -21054,7 +21054,7 @@
         </is>
       </c>
       <c r="B343" s="3" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
@@ -21701,7 +21701,7 @@
         </is>
       </c>
       <c r="B354" s="3" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
@@ -22299,7 +22299,7 @@
         </is>
       </c>
       <c r="B364" s="3" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
@@ -22594,7 +22594,7 @@
         </is>
       </c>
       <c r="B369" s="2" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
@@ -22889,7 +22889,7 @@
         </is>
       </c>
       <c r="B374" s="3" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
@@ -23188,7 +23188,7 @@
         </is>
       </c>
       <c r="B379" s="2" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
@@ -23487,7 +23487,7 @@
         </is>
       </c>
       <c r="B384" s="3" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
@@ -23806,7 +23806,7 @@
         </is>
       </c>
       <c r="B389" s="2" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
@@ -25874,7 +25874,7 @@
         </is>
       </c>
       <c r="B421" s="2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
@@ -27198,7 +27198,7 @@
         </is>
       </c>
       <c r="B441" s="2" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
@@ -27472,7 +27472,7 @@
         </is>
       </c>
       <c r="B445" s="3" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C445" s="3" t="inlineStr">
         <is>
@@ -28020,7 +28020,7 @@
         </is>
       </c>
       <c r="B453" s="3" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C453" s="3" t="inlineStr">
         <is>
@@ -28804,7 +28804,7 @@
         </is>
       </c>
       <c r="B465" s="3" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C465" s="3" t="inlineStr">
         <is>
@@ -29451,7 +29451,7 @@
         </is>
       </c>
       <c r="B476" s="3" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C476" s="3" t="inlineStr">
         <is>
@@ -30187,7 +30187,7 @@
         </is>
       </c>
       <c r="B488" s="3" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C488" s="3" t="inlineStr">
         <is>
@@ -30247,7 +30247,7 @@
       </c>
       <c r="O488" s="3" t="inlineStr">
         <is>
-          <t>Islam forbids alcohol, but drinking varies a lot across Muslim-majority countries: Bosnia and Herzegovina (5.87 litres of pure alcohol per adult) and Kazakhstan (4.52) drink far more than Turkey (1.69) or Pakistan (0.08), which is near the bottom of the world. Nigeria is 3.78 and the UAE 2.08. Muslim shares (Pew Research Center, 2020): Pakistan 96%, Turkey 97%, Kazakhstan 78%, UAE 73%, Nigeria 56% and Bosnia and Herzegovina 54%; other estimates put Nigeria closer to half. National averages include non-Muslims (and, in the UAE, a large expatriate population). WHO 2020 estimates for people aged 15+.</t>
+          <t>Islam forbids alcohol, but drinking varies a lot across Muslim-majority countries: Bosnia and Herzegovina (5.87 litres of pure alcohol per adult) and Kazakhstan (4.52) drink far more than Turkey (1.69) or Pakistan (0.08), which is near the bottom of the world. Nigeria is 3.78 and the UAE 2.08. Muslim shares (Pew Research Center, 2020): Pakistan 96%, Turkey 97%, Kazakhstan 78%, UAE 73%, Nigeria 56% and Bosnia and Herzegovina 54%. National averages include non-Muslims (and, in the UAE, a large expatriate population). WHO 2020 estimates for people aged 15+.</t>
         </is>
       </c>
       <c r="P488" s="3" t="inlineStr">
@@ -80861,7 +80861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -80880,6 +80880,7 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -80963,6 +80964,11 @@
           <t>flag_img</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -81035,6 +81041,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -81093,6 +81100,7 @@
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -81151,6 +81159,7 @@
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -81205,6 +81214,7 @@
       <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -81259,6 +81269,7 @@
       <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -81317,6 +81328,7 @@
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -81389,6 +81401,7 @@
       </c>
       <c r="O8" s="3" t="inlineStr"/>
       <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -81447,6 +81460,7 @@
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -81505,6 +81519,7 @@
           <t>flags/yug.svg</t>
         </is>
       </c>
+      <c r="Q10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -81563,6 +81578,7 @@
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -81617,6 +81633,7 @@
       <c r="N12" s="3" t="inlineStr"/>
       <c r="O12" s="3" t="inlineStr"/>
       <c r="P12" s="3" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -81671,6 +81688,7 @@
       <c r="N13" s="3" t="inlineStr"/>
       <c r="O13" s="3" t="inlineStr"/>
       <c r="P13" s="3" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -81729,9 +81747,785 @@
         </is>
       </c>
       <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>match-age-of-consent</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>⚖️</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Of Age</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Age of consent (with an adult who isn't a teacher or guardian)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>🇮🇹</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>14, or 16 if the adult is a teacher or guardian</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Italy's Penal Code (art. 609-quater) sets 14, rising to 16 when the older partner is a parent, guardian, teacher or anyone else the minor is entrusted to.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Wikipedia: Age of consent by country (Italian Penal Code art. 609-quater)</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/w/index.php?title=Age_of_consent_by_country&amp;oldid=1380397931</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>match-age-of-consent</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>🇺🇸</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>16, 17 or 18, depending on the state</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>There is no single national age: each state sets its own, 16 in many states and 17 or 18 in others (US Department of Health and Human Services guide to state laws).</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>US HHS (ASPE): Statutory Rape, A Guide to State Laws</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://aspe.hhs.gov/reports/state-laws</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>16 in some regions</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>match-age-of-consent</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>JPN</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>🇯🇵</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>16 nationally since 2023, though local youth ordinances are often seen as making it 18</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>In 2023 Japan raised its national age of consent from 13, unchanged since 1907, to 16. Regional ordinances banning 'lewd' acts with minors under 18 are often seen as raising it to 18 in practice.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>The Guardian (2023)</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theguardian.com/world/2023/jun/16/japan-raises-age-of-consent-from-13-to-16-in-reform-of-sex-crimes-law</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>match-age-of-consent</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>SVN</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>🇸🇮</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Slovenia</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Slovenia's Criminal Code sets the age of consent at 15, the same for everyone.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Wikipedia: Age of consent by country</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/w/index.php?title=Age_of_consent_by_country&amp;oldid=1380397931</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>match-age-of-consent</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>IRL</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>🇮🇪</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Ireland's Criminal Law (Sexual Offences) Act 2006 sets the age of consent at 17, one of the highest in Europe.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Irish Statute Book: Criminal Law (Sexual Offences) Act 2006</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.irishstatutebook.ie/eli/2006/act/15/enacted/en/html</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>match-age-of-consent</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Bahrain</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>BHR</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>🇧🇭</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Bahrain</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>21, unless the couple are married</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Bahrain's Penal Code (art. 345) punishes consensual sex with a female under 21; within marriage the age is 16.</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Penal Code of Bahrain (1976, as amended), via UNODC</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20150921155851/http://www.unodc.org/res/cld/document/bhr/1976/bahrain_penal_code_html/Bahrain_Penal_Code_1976.pdf</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>21 unless married</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>match-age-of-consent</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>MDG</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>🇲🇬</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>14, but 21 for same-sex relations</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Madagascar's Penal Code (art. 331) sets 14, but makes an 'indecent or unnatural act' with a same-sex partner under 21 a crime.</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Wikipedia: Age of consent by country (Madagascar Penal Code of 1972, art. 331)</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/w/index.php?title=Age_of_consent_by_country&amp;oldid=1380397931</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>14 for heterosexual and 21 for same-sex</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>match-child-rape-penalties</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>108</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>⚖️</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Hard Line</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Penalties in law for raping a child</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>JPN</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>🇯🇵</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>At least 5 years (up to 20) for a child under 16</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Penal Code art. 177 (revised 2023): non-consensual intercourse, which includes any intercourse with a child under 16 (13-15 if the adult is 5+ years older), carries a fixed term of at least 5 years; art. 12 caps fixed terms at 20.</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>e-Gov: Penal Code (Act No. 45 of 1907), art. 177</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>https://laws.e-gov.go.jp/law/140AC0000000045</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr"/>
+      <c r="P22" s="3" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>These are the penalties written in each country's law for the main child-rape offence, not the sentences courts actually hand down; age bands, aggravating factors and sentencing practice differ a lot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>match-child-rape-penalties</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>IND</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>🇮🇳</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>At least 20 years for a child under 16, and death is possible in aggravated cases</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>POCSO Act as amended in 2019: penetrative sexual assault on a child under 16 is at least 20 years up to life (s.4(2)); aggravated cases, e.g. a child under 12, are at least 20 years, life for the rest of natural life, or death (s.6).</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>PRS India: POCSO (Amendment) Bill 2019 summary</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>https://prsindia.org/billtrack/prs-products/prs-bill-summary-3279</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr"/>
+      <c r="P23" s="3" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>match-child-rape-penalties</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>PAK</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>🇵🇰</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Death or life in prison, and nothing lighter, for raping a minor</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Penal Code s.376(3) (added 2016): rape of a minor is punished with death or imprisonment for life, plus a fine. A 2021 bill's chemical-castration clause was dropped before it passed.</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Pakistan Penal Code s.376 (consolidated)</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>https://pakistankanoon.com/statutes.php/Pakistan-Penal-Code,-1860/Section-376/</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="inlineStr"/>
+      <c r="O24" s="3" t="inlineStr"/>
+      <c r="P24" s="3" t="inlineStr"/>
+      <c r="Q24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>match-child-rape-penalties</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>ISR</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>🇮🇱</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Up to 16 years for a child under 14, and at least a quarter of that unless the judge records special reasons</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Penal Law 5737-1977 s.345: sex with a child under 14 is rape even with 'consent' (16 years; 20 if aggravated, e.g. force on a child under 16). s.355 sets a minimum of one quarter of the maximum unless the court records special reasons. Death is not available.</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Penal Law 5737-1977 (English, via ICJ)</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.icj.org/wp-content/uploads/2013/05/Israel-Penal-Law-5737-1977-eng.pdf</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr"/>
+      <c r="O25" s="3" t="inlineStr"/>
+      <c r="P25" s="3" t="inlineStr"/>
+      <c r="Q25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>match-child-rape-penalties</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>NLD</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>🇳🇱</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Up to 15 years, or just a fine, for a child under 12; no minimum</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Criminal Code art. 250 (Sexual Offences Act, in force 1 July 2024): penetration of a child under 12 carries up to 15 years or a fifth-category fine, with no statutory minimum; ages 12-15 are up to 12 years (art. 248).</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>wetten.overheid.nl: Wetboek van Strafrecht, art. 248/250</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>https://wetten.overheid.nl/BWBR0001854/2024-10-01</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="inlineStr"/>
+      <c r="O26" s="3" t="inlineStr"/>
+      <c r="P26" s="3" t="inlineStr"/>
+      <c r="Q26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>match-child-rape-penalties</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>CHE</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>🇨🇭</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>1 to 5 years for sex with a child under 12 when no force is used</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Criminal Code art. 187 (revised 1 July 2024): a sexual act with a child under 12 is 1 to 5 years; under 16, up to 5 years or a monetary penalty. If force or coercion is used, rape (art. 190) is 1 to 10 years.</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Fedlex: Swiss Criminal Code, art. 187</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fedlex.admin.ch/eli/cc/54/757_781_799/en#art_187</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr"/>
+      <c r="O27" s="3" t="inlineStr"/>
+      <c r="P27" s="3" t="inlineStr"/>
+      <c r="Q27" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P14"/>
+  <autoFilter ref="A1:Q27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v12.2: three sex-ratio Rank its — Single Ladies!, Dating Odds, No Country for Old Men
CIA World Factbook males-per-female via Wikipedia oldid 1372609821, ranked as females per male.
Puerto Rico listed separately. Practice datasets added. aged-65 headline → Silver Wave. CNAME unchanged.
</commit_message>
<xml_diff>
--- a/puzzles.xlsx
+++ b/puzzles.xlsx
@@ -16,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOW TO EDIT" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'puzzles'!$A$1:$W$514</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'puzzles'!$A$1:$W$532</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'country_lists'!$A$1:$G$1009</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'country_info'!$A$1:$L$222</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'hint_bank'!$A$1:$H$181</definedName>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W514"/>
+  <dimension ref="A1:W532"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4443,7 +4443,7 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
@@ -5376,7 +5376,7 @@
         </is>
       </c>
       <c r="B85" s="3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
@@ -5868,7 +5868,7 @@
         </is>
       </c>
       <c r="B93" s="3" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
@@ -6530,7 +6530,7 @@
         </is>
       </c>
       <c r="B103" s="3" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
@@ -7795,7 +7795,7 @@
         </is>
       </c>
       <c r="B126" s="2" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
@@ -8021,7 +8021,7 @@
         </is>
       </c>
       <c r="B130" s="3" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
@@ -8247,7 +8247,7 @@
         </is>
       </c>
       <c r="B134" s="2" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         </is>
       </c>
       <c r="B139" s="3" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
@@ -9180,7 +9180,7 @@
         </is>
       </c>
       <c r="B149" s="3" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
@@ -9451,7 +9451,7 @@
         </is>
       </c>
       <c r="B154" s="2" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
         </is>
       </c>
       <c r="B174" s="2" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
@@ -11289,7 +11289,7 @@
         </is>
       </c>
       <c r="B184" s="2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
@@ -11911,7 +11911,7 @@
         </is>
       </c>
       <c r="B194" s="2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
@@ -12230,7 +12230,7 @@
         </is>
       </c>
       <c r="B199" s="3" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
@@ -12868,7 +12868,7 @@
         </is>
       </c>
       <c r="B209" s="3" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
@@ -13179,7 +13179,7 @@
         </is>
       </c>
       <c r="B214" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
@@ -13490,7 +13490,7 @@
         </is>
       </c>
       <c r="B219" s="3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
@@ -13817,7 +13817,7 @@
         </is>
       </c>
       <c r="B224" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
@@ -14156,7 +14156,7 @@
         </is>
       </c>
       <c r="B229" s="3" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
@@ -14487,7 +14487,7 @@
         </is>
       </c>
       <c r="B234" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
@@ -14798,7 +14798,7 @@
         </is>
       </c>
       <c r="B239" s="3" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
@@ -15109,7 +15109,7 @@
         </is>
       </c>
       <c r="B244" s="2" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
@@ -15428,7 +15428,7 @@
         </is>
       </c>
       <c r="B249" s="3" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
@@ -15800,7 +15800,7 @@
         </is>
       </c>
       <c r="B255" s="2" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
@@ -16099,7 +16099,7 @@
         </is>
       </c>
       <c r="B260" s="3" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
@@ -16746,7 +16746,7 @@
         </is>
       </c>
       <c r="B271" s="3" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
@@ -17041,7 +17041,7 @@
         </is>
       </c>
       <c r="B276" s="2" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
@@ -17340,7 +17340,7 @@
         </is>
       </c>
       <c r="B281" s="3" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
@@ -17639,7 +17639,7 @@
         </is>
       </c>
       <c r="B286" s="2" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
@@ -17958,7 +17958,7 @@
         </is>
       </c>
       <c r="B291" s="3" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
@@ -18330,7 +18330,7 @@
         </is>
       </c>
       <c r="B297" s="2" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
@@ -18629,7 +18629,7 @@
         </is>
       </c>
       <c r="B302" s="3" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
@@ -19272,7 +19272,7 @@
         </is>
       </c>
       <c r="B313" s="3" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
@@ -19567,7 +19567,7 @@
         </is>
       </c>
       <c r="B318" s="2" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
@@ -19866,7 +19866,7 @@
         </is>
       </c>
       <c r="B323" s="3" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
@@ -20165,7 +20165,7 @@
         </is>
       </c>
       <c r="B328" s="2" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
@@ -20464,7 +20464,7 @@
         </is>
       </c>
       <c r="B333" s="3" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
@@ -20759,7 +20759,7 @@
         </is>
       </c>
       <c r="B338" s="2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
@@ -21054,7 +21054,7 @@
         </is>
       </c>
       <c r="B343" s="3" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
@@ -21701,7 +21701,7 @@
         </is>
       </c>
       <c r="B354" s="3" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
@@ -22000,7 +22000,7 @@
         </is>
       </c>
       <c r="B359" s="2" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
@@ -22299,7 +22299,7 @@
         </is>
       </c>
       <c r="B364" s="3" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
@@ -22594,7 +22594,7 @@
         </is>
       </c>
       <c r="B369" s="2" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
@@ -22682,7 +22682,7 @@
       <c r="V369" s="2" t="inlineStr"/>
       <c r="W369" s="2" t="inlineStr">
         <is>
-          <t>No Country for Old Men</t>
+          <t>Silver Wave</t>
         </is>
       </c>
     </row>
@@ -22889,7 +22889,7 @@
         </is>
       </c>
       <c r="B374" s="3" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
@@ -23188,7 +23188,7 @@
         </is>
       </c>
       <c r="B379" s="2" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
@@ -23487,7 +23487,7 @@
         </is>
       </c>
       <c r="B384" s="3" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
@@ -23806,7 +23806,7 @@
         </is>
       </c>
       <c r="B389" s="2" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
@@ -24105,7 +24105,7 @@
         </is>
       </c>
       <c r="B394" s="3" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C394" s="3" t="inlineStr">
         <is>
@@ -24767,7 +24767,7 @@
         </is>
       </c>
       <c r="B404" s="3" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C404" s="3" t="inlineStr">
         <is>
@@ -25874,7 +25874,7 @@
         </is>
       </c>
       <c r="B421" s="2" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
@@ -26205,7 +26205,7 @@
         </is>
       </c>
       <c r="B426" s="3" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C426" s="3" t="inlineStr">
         <is>
@@ -26536,7 +26536,7 @@
         </is>
       </c>
       <c r="B431" s="2" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
@@ -26867,7 +26867,7 @@
         </is>
       </c>
       <c r="B436" s="3" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C436" s="3" t="inlineStr">
         <is>
@@ -27198,7 +27198,7 @@
         </is>
       </c>
       <c r="B441" s="2" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
@@ -27472,7 +27472,7 @@
         </is>
       </c>
       <c r="B445" s="3" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C445" s="3" t="inlineStr">
         <is>
@@ -27746,7 +27746,7 @@
         </is>
       </c>
       <c r="B449" s="2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
@@ -28020,7 +28020,7 @@
         </is>
       </c>
       <c r="B453" s="3" t="n">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C453" s="3" t="inlineStr">
         <is>
@@ -28804,7 +28804,7 @@
         </is>
       </c>
       <c r="B465" s="3" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C465" s="3" t="inlineStr">
         <is>
@@ -29451,7 +29451,7 @@
         </is>
       </c>
       <c r="B476" s="3" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C476" s="3" t="inlineStr">
         <is>
@@ -30187,7 +30187,7 @@
         </is>
       </c>
       <c r="B488" s="3" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C488" s="3" t="inlineStr">
         <is>
@@ -30555,7 +30555,7 @@
         </is>
       </c>
       <c r="B494" s="2" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
@@ -31488,7 +31488,7 @@
         </is>
       </c>
       <c r="B509" s="3" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C509" s="3" t="inlineStr">
         <is>
@@ -31845,8 +31845,1192 @@
       <c r="V514" s="3" t="inlineStr"/>
       <c r="W514" s="3" t="inlineStr"/>
     </row>
+    <row r="515">
+      <c r="A515" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64</t>
+        </is>
+      </c>
+      <c r="B515" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="C515" s="2" t="inlineStr">
+        <is>
+          <t>💃</t>
+        </is>
+      </c>
+      <c r="D515" s="2" t="inlineStr">
+        <is>
+          <t>Females per male, ages 15–64</t>
+        </is>
+      </c>
+      <c r="E515" s="2" t="inlineStr">
+        <is>
+          <t>Sex ratio ages 15–64, expressed as females per male (from World Factbook males-per-female via Wikipedia)</t>
+        </is>
+      </c>
+      <c r="F515" s="2" t="inlineStr">
+        <is>
+          <t>females per male</t>
+        </is>
+      </c>
+      <c r="G515" s="2" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H515" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I515" s="2" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="J515" s="2" t="inlineStr">
+        <is>
+          <t>🇭🇰</t>
+        </is>
+      </c>
+      <c r="K515" s="2" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="L515" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M515" s="2" t="inlineStr">
+        <is>
+          <t>Wikipedia / CIA World Factbook: List of countries by sex ratio</t>
+        </is>
+      </c>
+      <c r="N515" s="2" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_countries_by_sex_ratio?oldid=1372609821</t>
+        </is>
+      </c>
+      <c r="O515" s="2" t="inlineStr">
+        <is>
+          <t>World Factbook male-to-female ratios for ages 15–64, via Wikipedia (rev 1372609821). Ranked as females per male (1 ÷ Factbook ratio). Qatar and similar Gulf states have many more men because of migrant labour. Caveat: Factbook estimates; national censuses can differ.</t>
+        </is>
+      </c>
+      <c r="P515" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q515" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R515" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S515" s="2" t="inlineStr">
+        <is>
+          <t>heart</t>
+        </is>
+      </c>
+      <c r="T515" s="2" t="inlineStr"/>
+      <c r="U515" s="2" t="inlineStr">
+        <is>
+          <t>cia-sex-ratio-15-64</t>
+        </is>
+      </c>
+      <c r="V515" s="2" t="inlineStr">
+        <is>
+          <t>Females per Male (15–64)</t>
+        </is>
+      </c>
+      <c r="W515" s="2" t="inlineStr">
+        <is>
+          <t>Single Ladies!</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64</t>
+        </is>
+      </c>
+      <c r="B516" s="2" t="inlineStr"/>
+      <c r="C516" s="2" t="inlineStr"/>
+      <c r="D516" s="2" t="inlineStr"/>
+      <c r="E516" s="2" t="inlineStr"/>
+      <c r="F516" s="2" t="inlineStr"/>
+      <c r="G516" s="2" t="inlineStr"/>
+      <c r="H516" s="2" t="inlineStr"/>
+      <c r="I516" s="2" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="J516" s="2" t="inlineStr">
+        <is>
+          <t>🇷🇺</t>
+        </is>
+      </c>
+      <c r="K516" s="2" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
+      </c>
+      <c r="L516" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M516" s="2" t="inlineStr"/>
+      <c r="N516" s="2" t="inlineStr"/>
+      <c r="O516" s="2" t="inlineStr"/>
+      <c r="P516" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="Q516" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R516" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S516" s="2" t="inlineStr"/>
+      <c r="T516" s="2" t="inlineStr"/>
+      <c r="U516" s="2" t="inlineStr"/>
+      <c r="V516" s="2" t="inlineStr"/>
+      <c r="W516" s="2" t="inlineStr"/>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64</t>
+        </is>
+      </c>
+      <c r="B517" s="2" t="inlineStr"/>
+      <c r="C517" s="2" t="inlineStr"/>
+      <c r="D517" s="2" t="inlineStr"/>
+      <c r="E517" s="2" t="inlineStr"/>
+      <c r="F517" s="2" t="inlineStr"/>
+      <c r="G517" s="2" t="inlineStr"/>
+      <c r="H517" s="2" t="inlineStr"/>
+      <c r="I517" s="2" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="J517" s="2" t="inlineStr">
+        <is>
+          <t>🇹🇭</t>
+        </is>
+      </c>
+      <c r="K517" s="2" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="L517" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M517" s="2" t="inlineStr"/>
+      <c r="N517" s="2" t="inlineStr"/>
+      <c r="O517" s="2" t="inlineStr"/>
+      <c r="P517" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="Q517" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R517" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S517" s="2" t="inlineStr"/>
+      <c r="T517" s="2" t="inlineStr"/>
+      <c r="U517" s="2" t="inlineStr"/>
+      <c r="V517" s="2" t="inlineStr"/>
+      <c r="W517" s="2" t="inlineStr"/>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64</t>
+        </is>
+      </c>
+      <c r="B518" s="2" t="inlineStr"/>
+      <c r="C518" s="2" t="inlineStr"/>
+      <c r="D518" s="2" t="inlineStr"/>
+      <c r="E518" s="2" t="inlineStr"/>
+      <c r="F518" s="2" t="inlineStr"/>
+      <c r="G518" s="2" t="inlineStr"/>
+      <c r="H518" s="2" t="inlineStr"/>
+      <c r="I518" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="J518" s="2" t="inlineStr">
+        <is>
+          <t>🇺🇸</t>
+        </is>
+      </c>
+      <c r="K518" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="L518" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M518" s="2" t="inlineStr"/>
+      <c r="N518" s="2" t="inlineStr"/>
+      <c r="O518" s="2" t="inlineStr"/>
+      <c r="P518" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="Q518" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R518" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S518" s="2" t="inlineStr"/>
+      <c r="T518" s="2" t="inlineStr"/>
+      <c r="U518" s="2" t="inlineStr"/>
+      <c r="V518" s="2" t="inlineStr"/>
+      <c r="W518" s="2" t="inlineStr"/>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64</t>
+        </is>
+      </c>
+      <c r="B519" s="2" t="inlineStr"/>
+      <c r="C519" s="2" t="inlineStr"/>
+      <c r="D519" s="2" t="inlineStr"/>
+      <c r="E519" s="2" t="inlineStr"/>
+      <c r="F519" s="2" t="inlineStr"/>
+      <c r="G519" s="2" t="inlineStr"/>
+      <c r="H519" s="2" t="inlineStr"/>
+      <c r="I519" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J519" s="2" t="inlineStr">
+        <is>
+          <t>🇮🇳</t>
+        </is>
+      </c>
+      <c r="K519" s="2" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="L519" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M519" s="2" t="inlineStr"/>
+      <c r="N519" s="2" t="inlineStr"/>
+      <c r="O519" s="2" t="inlineStr"/>
+      <c r="P519" s="2" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="Q519" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R519" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S519" s="2" t="inlineStr"/>
+      <c r="T519" s="2" t="inlineStr"/>
+      <c r="U519" s="2" t="inlineStr"/>
+      <c r="V519" s="2" t="inlineStr"/>
+      <c r="W519" s="2" t="inlineStr"/>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64</t>
+        </is>
+      </c>
+      <c r="B520" s="2" t="inlineStr"/>
+      <c r="C520" s="2" t="inlineStr"/>
+      <c r="D520" s="2" t="inlineStr"/>
+      <c r="E520" s="2" t="inlineStr"/>
+      <c r="F520" s="2" t="inlineStr"/>
+      <c r="G520" s="2" t="inlineStr"/>
+      <c r="H520" s="2" t="inlineStr"/>
+      <c r="I520" s="2" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="J520" s="2" t="inlineStr">
+        <is>
+          <t>🇶🇦</t>
+        </is>
+      </c>
+      <c r="K520" s="2" t="inlineStr">
+        <is>
+          <t>0.23</t>
+        </is>
+      </c>
+      <c r="L520" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M520" s="2" t="inlineStr"/>
+      <c r="N520" s="2" t="inlineStr"/>
+      <c r="O520" s="2" t="inlineStr"/>
+      <c r="P520" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="Q520" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R520" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S520" s="2" t="inlineStr"/>
+      <c r="T520" s="2" t="inlineStr"/>
+      <c r="U520" s="2" t="inlineStr"/>
+      <c r="V520" s="2" t="inlineStr"/>
+      <c r="W520" s="2" t="inlineStr"/>
+    </row>
+    <row r="521">
+      <c r="A521" s="3" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64-b</t>
+        </is>
+      </c>
+      <c r="B521" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="C521" s="3" t="inlineStr">
+        <is>
+          <t>💘</t>
+        </is>
+      </c>
+      <c r="D521" s="3" t="inlineStr">
+        <is>
+          <t>Females per male, ages 15–64</t>
+        </is>
+      </c>
+      <c r="E521" s="3" t="inlineStr">
+        <is>
+          <t>Sex ratio ages 15–64, expressed as females per male (from World Factbook males-per-female via Wikipedia)</t>
+        </is>
+      </c>
+      <c r="F521" s="3" t="inlineStr">
+        <is>
+          <t>females per male</t>
+        </is>
+      </c>
+      <c r="G521" s="3" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H521" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I521" s="3" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="J521" s="3" t="inlineStr">
+        <is>
+          <t>🇵🇷</t>
+        </is>
+      </c>
+      <c r="K521" s="3" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="L521" s="3" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M521" s="3" t="inlineStr">
+        <is>
+          <t>Wikipedia / CIA World Factbook: List of countries by sex ratio</t>
+        </is>
+      </c>
+      <c r="N521" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_countries_by_sex_ratio?oldid=1372609821</t>
+        </is>
+      </c>
+      <c r="O521" s="3" t="inlineStr">
+        <is>
+          <t>World Factbook male-to-female ratios for ages 15–64, via Wikipedia (rev 1372609821). Ranked as females per male (1 ÷ Factbook ratio). Qatar and similar Gulf states have many more men because of migrant labour. Caveat: Factbook estimates; national censuses can differ.</t>
+        </is>
+      </c>
+      <c r="P521" s="3" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="Q521" s="3" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R521" s="3" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S521" s="3" t="inlineStr">
+        <is>
+          <t>heart</t>
+        </is>
+      </c>
+      <c r="T521" s="3" t="inlineStr"/>
+      <c r="U521" s="3" t="inlineStr">
+        <is>
+          <t>cia-sex-ratio-15-64</t>
+        </is>
+      </c>
+      <c r="V521" s="3" t="inlineStr">
+        <is>
+          <t>Females per Male (15–64)</t>
+        </is>
+      </c>
+      <c r="W521" s="3" t="inlineStr">
+        <is>
+          <t>Dating Odds</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="3" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64-b</t>
+        </is>
+      </c>
+      <c r="B522" s="3" t="inlineStr"/>
+      <c r="C522" s="3" t="inlineStr"/>
+      <c r="D522" s="3" t="inlineStr"/>
+      <c r="E522" s="3" t="inlineStr"/>
+      <c r="F522" s="3" t="inlineStr"/>
+      <c r="G522" s="3" t="inlineStr"/>
+      <c r="H522" s="3" t="inlineStr"/>
+      <c r="I522" s="3" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="J522" s="3" t="inlineStr">
+        <is>
+          <t>🇮🇪</t>
+        </is>
+      </c>
+      <c r="K522" s="3" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="L522" s="3" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M522" s="3" t="inlineStr"/>
+      <c r="N522" s="3" t="inlineStr"/>
+      <c r="O522" s="3" t="inlineStr"/>
+      <c r="P522" s="3" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="Q522" s="3" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R522" s="3" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S522" s="3" t="inlineStr"/>
+      <c r="T522" s="3" t="inlineStr"/>
+      <c r="U522" s="3" t="inlineStr"/>
+      <c r="V522" s="3" t="inlineStr"/>
+      <c r="W522" s="3" t="inlineStr"/>
+    </row>
+    <row r="523">
+      <c r="A523" s="3" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64-b</t>
+        </is>
+      </c>
+      <c r="B523" s="3" t="inlineStr"/>
+      <c r="C523" s="3" t="inlineStr"/>
+      <c r="D523" s="3" t="inlineStr"/>
+      <c r="E523" s="3" t="inlineStr"/>
+      <c r="F523" s="3" t="inlineStr"/>
+      <c r="G523" s="3" t="inlineStr"/>
+      <c r="H523" s="3" t="inlineStr"/>
+      <c r="I523" s="3" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="J523" s="3" t="inlineStr">
+        <is>
+          <t>🇬🇧</t>
+        </is>
+      </c>
+      <c r="K523" s="3" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="L523" s="3" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M523" s="3" t="inlineStr"/>
+      <c r="N523" s="3" t="inlineStr"/>
+      <c r="O523" s="3" t="inlineStr"/>
+      <c r="P523" s="3" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="Q523" s="3" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R523" s="3" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S523" s="3" t="inlineStr"/>
+      <c r="T523" s="3" t="inlineStr"/>
+      <c r="U523" s="3" t="inlineStr"/>
+      <c r="V523" s="3" t="inlineStr"/>
+      <c r="W523" s="3" t="inlineStr"/>
+    </row>
+    <row r="524">
+      <c r="A524" s="3" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64-b</t>
+        </is>
+      </c>
+      <c r="B524" s="3" t="inlineStr"/>
+      <c r="C524" s="3" t="inlineStr"/>
+      <c r="D524" s="3" t="inlineStr"/>
+      <c r="E524" s="3" t="inlineStr"/>
+      <c r="F524" s="3" t="inlineStr"/>
+      <c r="G524" s="3" t="inlineStr"/>
+      <c r="H524" s="3" t="inlineStr"/>
+      <c r="I524" s="3" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="J524" s="3" t="inlineStr">
+        <is>
+          <t>🇨🇳</t>
+        </is>
+      </c>
+      <c r="K524" s="3" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="L524" s="3" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M524" s="3" t="inlineStr"/>
+      <c r="N524" s="3" t="inlineStr"/>
+      <c r="O524" s="3" t="inlineStr"/>
+      <c r="P524" s="3" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="Q524" s="3" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R524" s="3" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S524" s="3" t="inlineStr"/>
+      <c r="T524" s="3" t="inlineStr"/>
+      <c r="U524" s="3" t="inlineStr"/>
+      <c r="V524" s="3" t="inlineStr"/>
+      <c r="W524" s="3" t="inlineStr"/>
+    </row>
+    <row r="525">
+      <c r="A525" s="3" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64-b</t>
+        </is>
+      </c>
+      <c r="B525" s="3" t="inlineStr"/>
+      <c r="C525" s="3" t="inlineStr"/>
+      <c r="D525" s="3" t="inlineStr"/>
+      <c r="E525" s="3" t="inlineStr"/>
+      <c r="F525" s="3" t="inlineStr"/>
+      <c r="G525" s="3" t="inlineStr"/>
+      <c r="H525" s="3" t="inlineStr"/>
+      <c r="I525" s="3" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="J525" s="3" t="inlineStr">
+        <is>
+          <t>🇰🇷</t>
+        </is>
+      </c>
+      <c r="K525" s="3" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="L525" s="3" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M525" s="3" t="inlineStr"/>
+      <c r="N525" s="3" t="inlineStr"/>
+      <c r="O525" s="3" t="inlineStr"/>
+      <c r="P525" s="3" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+      <c r="Q525" s="3" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R525" s="3" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S525" s="3" t="inlineStr"/>
+      <c r="T525" s="3" t="inlineStr"/>
+      <c r="U525" s="3" t="inlineStr"/>
+      <c r="V525" s="3" t="inlineStr"/>
+      <c r="W525" s="3" t="inlineStr"/>
+    </row>
+    <row r="526">
+      <c r="A526" s="3" t="inlineStr">
+        <is>
+          <t>sex-ratio-15-64-b</t>
+        </is>
+      </c>
+      <c r="B526" s="3" t="inlineStr"/>
+      <c r="C526" s="3" t="inlineStr"/>
+      <c r="D526" s="3" t="inlineStr"/>
+      <c r="E526" s="3" t="inlineStr"/>
+      <c r="F526" s="3" t="inlineStr"/>
+      <c r="G526" s="3" t="inlineStr"/>
+      <c r="H526" s="3" t="inlineStr"/>
+      <c r="I526" s="3" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="J526" s="3" t="inlineStr">
+        <is>
+          <t>🇸🇦</t>
+        </is>
+      </c>
+      <c r="K526" s="3" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="L526" s="3" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M526" s="3" t="inlineStr"/>
+      <c r="N526" s="3" t="inlineStr"/>
+      <c r="O526" s="3" t="inlineStr"/>
+      <c r="P526" s="3" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="Q526" s="3" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R526" s="3" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S526" s="3" t="inlineStr"/>
+      <c r="T526" s="3" t="inlineStr"/>
+      <c r="U526" s="3" t="inlineStr"/>
+      <c r="V526" s="3" t="inlineStr"/>
+      <c r="W526" s="3" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-65</t>
+        </is>
+      </c>
+      <c r="B527" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C527" s="2" t="inlineStr">
+        <is>
+          <t>👵</t>
+        </is>
+      </c>
+      <c r="D527" s="2" t="inlineStr">
+        <is>
+          <t>Females per Male (65+)</t>
+        </is>
+      </c>
+      <c r="E527" s="2" t="inlineStr">
+        <is>
+          <t>Sex ratio ages 65+, expressed as females per male (from World Factbook males-per-female via Wikipedia)</t>
+        </is>
+      </c>
+      <c r="F527" s="2" t="inlineStr">
+        <is>
+          <t>females per male</t>
+        </is>
+      </c>
+      <c r="G527" s="2" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H527" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I527" s="2" t="inlineStr">
+        <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="J527" s="2" t="inlineStr">
+        <is>
+          <t>🇺🇦</t>
+        </is>
+      </c>
+      <c r="K527" s="2" t="inlineStr">
+        <is>
+          <t>1.89</t>
+        </is>
+      </c>
+      <c r="L527" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M527" s="2" t="inlineStr">
+        <is>
+          <t>Wikipedia / CIA World Factbook: List of countries by sex ratio</t>
+        </is>
+      </c>
+      <c r="N527" s="2" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_countries_by_sex_ratio?oldid=1372609821</t>
+        </is>
+      </c>
+      <c r="O527" s="2" t="inlineStr">
+        <is>
+          <t>World Factbook male-to-female ratios for ages 65+, via Wikipedia (rev 1372609821). Ranked as females per male. Most countries have more older women than older men; the Gulf is an exception where working-age male migration still shapes the older cohorts. Caveat: Factbook estimates.</t>
+        </is>
+      </c>
+      <c r="P527" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="Q527" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R527" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S527" s="2" t="inlineStr">
+        <is>
+          <t>cake</t>
+        </is>
+      </c>
+      <c r="T527" s="2" t="inlineStr"/>
+      <c r="U527" s="2" t="inlineStr">
+        <is>
+          <t>cia-sex-ratio-65</t>
+        </is>
+      </c>
+      <c r="V527" s="2" t="inlineStr"/>
+      <c r="W527" s="2" t="inlineStr">
+        <is>
+          <t>No Country for Old Men</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-65</t>
+        </is>
+      </c>
+      <c r="B528" s="2" t="inlineStr"/>
+      <c r="C528" s="2" t="inlineStr"/>
+      <c r="D528" s="2" t="inlineStr"/>
+      <c r="E528" s="2" t="inlineStr"/>
+      <c r="F528" s="2" t="inlineStr"/>
+      <c r="G528" s="2" t="inlineStr"/>
+      <c r="H528" s="2" t="inlineStr"/>
+      <c r="I528" s="2" t="inlineStr">
+        <is>
+          <t>Cambodia</t>
+        </is>
+      </c>
+      <c r="J528" s="2" t="inlineStr">
+        <is>
+          <t>🇰🇭</t>
+        </is>
+      </c>
+      <c r="K528" s="2" t="inlineStr">
+        <is>
+          <t>1.82</t>
+        </is>
+      </c>
+      <c r="L528" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M528" s="2" t="inlineStr"/>
+      <c r="N528" s="2" t="inlineStr"/>
+      <c r="O528" s="2" t="inlineStr"/>
+      <c r="P528" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q528" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R528" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S528" s="2" t="inlineStr"/>
+      <c r="T528" s="2" t="inlineStr"/>
+      <c r="U528" s="2" t="inlineStr"/>
+      <c r="V528" s="2" t="inlineStr"/>
+      <c r="W528" s="2" t="inlineStr"/>
+    </row>
+    <row r="529">
+      <c r="A529" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-65</t>
+        </is>
+      </c>
+      <c r="B529" s="2" t="inlineStr"/>
+      <c r="C529" s="2" t="inlineStr"/>
+      <c r="D529" s="2" t="inlineStr"/>
+      <c r="E529" s="2" t="inlineStr"/>
+      <c r="F529" s="2" t="inlineStr"/>
+      <c r="G529" s="2" t="inlineStr"/>
+      <c r="H529" s="2" t="inlineStr"/>
+      <c r="I529" s="2" t="inlineStr">
+        <is>
+          <t>North Korea</t>
+        </is>
+      </c>
+      <c r="J529" s="2" t="inlineStr">
+        <is>
+          <t>🇰🇵</t>
+        </is>
+      </c>
+      <c r="K529" s="2" t="inlineStr">
+        <is>
+          <t>1.69</t>
+        </is>
+      </c>
+      <c r="L529" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M529" s="2" t="inlineStr"/>
+      <c r="N529" s="2" t="inlineStr"/>
+      <c r="O529" s="2" t="inlineStr"/>
+      <c r="P529" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="Q529" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R529" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S529" s="2" t="inlineStr"/>
+      <c r="T529" s="2" t="inlineStr"/>
+      <c r="U529" s="2" t="inlineStr"/>
+      <c r="V529" s="2" t="inlineStr"/>
+      <c r="W529" s="2" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-65</t>
+        </is>
+      </c>
+      <c r="B530" s="2" t="inlineStr"/>
+      <c r="C530" s="2" t="inlineStr"/>
+      <c r="D530" s="2" t="inlineStr"/>
+      <c r="E530" s="2" t="inlineStr"/>
+      <c r="F530" s="2" t="inlineStr"/>
+      <c r="G530" s="2" t="inlineStr"/>
+      <c r="H530" s="2" t="inlineStr"/>
+      <c r="I530" s="2" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="J530" s="2" t="inlineStr">
+        <is>
+          <t>🇵🇹</t>
+        </is>
+      </c>
+      <c r="K530" s="2" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="L530" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M530" s="2" t="inlineStr"/>
+      <c r="N530" s="2" t="inlineStr"/>
+      <c r="O530" s="2" t="inlineStr"/>
+      <c r="P530" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="Q530" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R530" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S530" s="2" t="inlineStr"/>
+      <c r="T530" s="2" t="inlineStr"/>
+      <c r="U530" s="2" t="inlineStr"/>
+      <c r="V530" s="2" t="inlineStr"/>
+      <c r="W530" s="2" t="inlineStr"/>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-65</t>
+        </is>
+      </c>
+      <c r="B531" s="2" t="inlineStr"/>
+      <c r="C531" s="2" t="inlineStr"/>
+      <c r="D531" s="2" t="inlineStr"/>
+      <c r="E531" s="2" t="inlineStr"/>
+      <c r="F531" s="2" t="inlineStr"/>
+      <c r="G531" s="2" t="inlineStr"/>
+      <c r="H531" s="2" t="inlineStr"/>
+      <c r="I531" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="J531" s="2" t="inlineStr">
+        <is>
+          <t>🇺🇸</t>
+        </is>
+      </c>
+      <c r="K531" s="2" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="L531" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M531" s="2" t="inlineStr"/>
+      <c r="N531" s="2" t="inlineStr"/>
+      <c r="O531" s="2" t="inlineStr"/>
+      <c r="P531" s="2" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="Q531" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R531" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S531" s="2" t="inlineStr"/>
+      <c r="T531" s="2" t="inlineStr"/>
+      <c r="U531" s="2" t="inlineStr"/>
+      <c r="V531" s="2" t="inlineStr"/>
+      <c r="W531" s="2" t="inlineStr"/>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="inlineStr">
+        <is>
+          <t>sex-ratio-65</t>
+        </is>
+      </c>
+      <c r="B532" s="2" t="inlineStr"/>
+      <c r="C532" s="2" t="inlineStr"/>
+      <c r="D532" s="2" t="inlineStr"/>
+      <c r="E532" s="2" t="inlineStr"/>
+      <c r="F532" s="2" t="inlineStr"/>
+      <c r="G532" s="2" t="inlineStr"/>
+      <c r="H532" s="2" t="inlineStr"/>
+      <c r="I532" s="2" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="J532" s="2" t="inlineStr">
+        <is>
+          <t>🇦🇪</t>
+        </is>
+      </c>
+      <c r="K532" s="2" t="inlineStr">
+        <is>
+          <t>0.31</t>
+        </is>
+      </c>
+      <c r="L532" s="2" t="inlineStr">
+        <is>
+          <t>Factbook / Wikipedia 2026</t>
+        </is>
+      </c>
+      <c r="M532" s="2" t="inlineStr"/>
+      <c r="N532" s="2" t="inlineStr"/>
+      <c r="O532" s="2" t="inlineStr"/>
+      <c r="P532" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="Q532" s="2" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="R532" s="2" t="inlineStr">
+        <is>
+          <t>listed places</t>
+        </is>
+      </c>
+      <c r="S532" s="2" t="inlineStr"/>
+      <c r="T532" s="2" t="inlineStr"/>
+      <c r="U532" s="2" t="inlineStr"/>
+      <c r="V532" s="2" t="inlineStr"/>
+      <c r="W532" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W514"/>
+  <autoFilter ref="A1:W532"/>
   <dataValidations count="2">
     <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"top,bottom"</formula1>
@@ -79688,7 +80872,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -79901,7 +81085,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -79972,7 +81156,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -80410,7 +81594,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -80715,7 +81899,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -81083,7 +82267,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
v12.2: Equaldex Legal/Opinion Rank its + sex-ratio as women per 100 men
Four sensitive Equaldex puzzles (Protect the Gays, On the Books, Why are
you gay?, Asking for a Friend) from equaldex.com/equality-index (scraped
2026-10-23). Sex-ratio three show women per 100 men. Schedule 120; no
back-to-back sensitive.
</commit_message>
<xml_diff>
--- a/puzzles.xlsx
+++ b/puzzles.xlsx
@@ -16,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOW TO EDIT" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'puzzles'!$A$1:$W$532</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'puzzles'!$A$1:$W$556</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'country_lists'!$A$1:$G$1009</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'country_info'!$A$1:$L$222</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'hint_bank'!$A$1:$H$181</definedName>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W532"/>
+  <dimension ref="A1:W556"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4443,7 +4443,7 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
@@ -5376,7 +5376,7 @@
         </is>
       </c>
       <c r="B85" s="3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
@@ -5868,7 +5868,7 @@
         </is>
       </c>
       <c r="B93" s="3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
@@ -6530,7 +6530,7 @@
         </is>
       </c>
       <c r="B103" s="3" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
@@ -7795,7 +7795,7 @@
         </is>
       </c>
       <c r="B126" s="2" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
@@ -8021,7 +8021,7 @@
         </is>
       </c>
       <c r="B130" s="3" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
@@ -8247,7 +8247,7 @@
         </is>
       </c>
       <c r="B134" s="2" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         </is>
       </c>
       <c r="B139" s="3" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
@@ -9180,7 +9180,7 @@
         </is>
       </c>
       <c r="B149" s="3" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
@@ -9451,7 +9451,7 @@
         </is>
       </c>
       <c r="B154" s="2" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10655,7 @@
         </is>
       </c>
       <c r="B174" s="2" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
@@ -11289,7 +11289,7 @@
         </is>
       </c>
       <c r="B184" s="2" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
@@ -11911,7 +11911,7 @@
         </is>
       </c>
       <c r="B194" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
@@ -12230,7 +12230,7 @@
         </is>
       </c>
       <c r="B199" s="3" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
@@ -12868,7 +12868,7 @@
         </is>
       </c>
       <c r="B209" s="3" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
@@ -13179,7 +13179,7 @@
         </is>
       </c>
       <c r="B214" s="2" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
@@ -13490,7 +13490,7 @@
         </is>
       </c>
       <c r="B219" s="3" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
@@ -13817,7 +13817,7 @@
         </is>
       </c>
       <c r="B224" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
@@ -14156,7 +14156,7 @@
         </is>
       </c>
       <c r="B229" s="3" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
@@ -14487,7 +14487,7 @@
         </is>
       </c>
       <c r="B234" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
@@ -14798,7 +14798,7 @@
         </is>
       </c>
       <c r="B239" s="3" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
@@ -15109,7 +15109,7 @@
         </is>
       </c>
       <c r="B244" s="2" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
@@ -15428,7 +15428,7 @@
         </is>
       </c>
       <c r="B249" s="3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
@@ -15800,7 +15800,7 @@
         </is>
       </c>
       <c r="B255" s="2" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
@@ -16099,7 +16099,7 @@
         </is>
       </c>
       <c r="B260" s="3" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
@@ -16746,7 +16746,7 @@
         </is>
       </c>
       <c r="B271" s="3" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
@@ -17041,7 +17041,7 @@
         </is>
       </c>
       <c r="B276" s="2" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
@@ -17340,7 +17340,7 @@
         </is>
       </c>
       <c r="B281" s="3" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
@@ -17639,7 +17639,7 @@
         </is>
       </c>
       <c r="B286" s="2" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
@@ -17958,7 +17958,7 @@
         </is>
       </c>
       <c r="B291" s="3" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
@@ -18330,7 +18330,7 @@
         </is>
       </c>
       <c r="B297" s="2" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
@@ -18629,7 +18629,7 @@
         </is>
       </c>
       <c r="B302" s="3" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
@@ -19272,7 +19272,7 @@
         </is>
       </c>
       <c r="B313" s="3" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
@@ -19567,7 +19567,7 @@
         </is>
       </c>
       <c r="B318" s="2" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
@@ -19866,7 +19866,7 @@
         </is>
       </c>
       <c r="B323" s="3" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
@@ -20165,7 +20165,7 @@
         </is>
       </c>
       <c r="B328" s="2" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
@@ -20464,7 +20464,7 @@
         </is>
       </c>
       <c r="B333" s="3" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
@@ -20759,7 +20759,7 @@
         </is>
       </c>
       <c r="B338" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
@@ -21054,7 +21054,7 @@
         </is>
       </c>
       <c r="B343" s="3" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
@@ -21701,7 +21701,7 @@
         </is>
       </c>
       <c r="B354" s="3" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
@@ -22000,7 +22000,7 @@
         </is>
       </c>
       <c r="B359" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
@@ -22299,7 +22299,7 @@
         </is>
       </c>
       <c r="B364" s="3" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
@@ -22594,7 +22594,7 @@
         </is>
       </c>
       <c r="B369" s="2" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
@@ -22889,7 +22889,7 @@
         </is>
       </c>
       <c r="B374" s="3" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
@@ -23188,7 +23188,7 @@
         </is>
       </c>
       <c r="B379" s="2" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
@@ -23487,7 +23487,7 @@
         </is>
       </c>
       <c r="B384" s="3" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
@@ -23806,7 +23806,7 @@
         </is>
       </c>
       <c r="B389" s="2" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
@@ -24105,7 +24105,7 @@
         </is>
       </c>
       <c r="B394" s="3" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C394" s="3" t="inlineStr">
         <is>
@@ -24767,7 +24767,7 @@
         </is>
       </c>
       <c r="B404" s="3" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C404" s="3" t="inlineStr">
         <is>
@@ -25874,7 +25874,7 @@
         </is>
       </c>
       <c r="B421" s="2" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
@@ -26205,7 +26205,7 @@
         </is>
       </c>
       <c r="B426" s="3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C426" s="3" t="inlineStr">
         <is>
@@ -26536,7 +26536,7 @@
         </is>
       </c>
       <c r="B431" s="2" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
@@ -26867,7 +26867,7 @@
         </is>
       </c>
       <c r="B436" s="3" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C436" s="3" t="inlineStr">
         <is>
@@ -27198,7 +27198,7 @@
         </is>
       </c>
       <c r="B441" s="2" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
@@ -27472,7 +27472,7 @@
         </is>
       </c>
       <c r="B445" s="3" t="n">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C445" s="3" t="inlineStr">
         <is>
@@ -27746,7 +27746,7 @@
         </is>
       </c>
       <c r="B449" s="2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
@@ -28020,7 +28020,7 @@
         </is>
       </c>
       <c r="B453" s="3" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C453" s="3" t="inlineStr">
         <is>
@@ -28804,7 +28804,7 @@
         </is>
       </c>
       <c r="B465" s="3" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C465" s="3" t="inlineStr">
         <is>
@@ -29451,7 +29451,7 @@
         </is>
       </c>
       <c r="B476" s="3" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C476" s="3" t="inlineStr">
         <is>
@@ -30187,7 +30187,7 @@
         </is>
       </c>
       <c r="B488" s="3" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C488" s="3" t="inlineStr">
         <is>
@@ -30555,7 +30555,7 @@
         </is>
       </c>
       <c r="B494" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
@@ -31488,7 +31488,7 @@
         </is>
       </c>
       <c r="B509" s="3" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C509" s="3" t="inlineStr">
         <is>
@@ -31861,17 +31861,17 @@
       </c>
       <c r="D515" s="2" t="inlineStr">
         <is>
-          <t>Females per male, ages 15–64</t>
+          <t>Women per 100 Men (15–64)</t>
         </is>
       </c>
       <c r="E515" s="2" t="inlineStr">
         <is>
-          <t>Sex ratio ages 15–64, expressed as females per male (from World Factbook males-per-female via Wikipedia)</t>
+          <t>Sex ratio ages 15–64, women per 100 men (from World Factbook males-per-female via Wikipedia; = 100 ÷ Factbook ratio)</t>
         </is>
       </c>
       <c r="F515" s="2" t="inlineStr">
         <is>
-          <t>females per male</t>
+          <t>women per 100 men</t>
         </is>
       </c>
       <c r="G515" s="2" t="inlineStr">
@@ -31896,7 +31896,7 @@
       </c>
       <c r="K515" s="2" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>123</t>
         </is>
       </c>
       <c r="L515" s="2" t="inlineStr">
@@ -31916,7 +31916,7 @@
       </c>
       <c r="O515" s="2" t="inlineStr">
         <is>
-          <t>World Factbook male-to-female ratios for ages 15–64, via Wikipedia (rev 1372609821). Ranked as females per male (1 ÷ Factbook ratio). Qatar and similar Gulf states have many more men because of migrant labour. Caveat: Factbook estimates; national censuses can differ.</t>
+          <t>World Factbook male-to-female ratios for ages 15–64, via Wikipedia (rev 1372609821). Ranked as women per 100 men (100 ÷ Factbook males-per-female ratio). Qatar and similar Gulf states have many more men because of migrant labour. Caveat: Factbook estimates; national censuses can differ.</t>
         </is>
       </c>
       <c r="P515" s="2" t="inlineStr">
@@ -31947,7 +31947,7 @@
       </c>
       <c r="V515" s="2" t="inlineStr">
         <is>
-          <t>Females per Male (15–64)</t>
+          <t>Women per 100 Men (15–64)</t>
         </is>
       </c>
       <c r="W515" s="2" t="inlineStr">
@@ -31981,7 +31981,7 @@
       </c>
       <c r="K516" s="2" t="inlineStr">
         <is>
-          <t>1.05</t>
+          <t>105</t>
         </is>
       </c>
       <c r="L516" s="2" t="inlineStr">
@@ -32038,7 +32038,7 @@
       </c>
       <c r="K517" s="2" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>104</t>
         </is>
       </c>
       <c r="L517" s="2" t="inlineStr">
@@ -32095,7 +32095,7 @@
       </c>
       <c r="K518" s="2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>100</t>
         </is>
       </c>
       <c r="L518" s="2" t="inlineStr">
@@ -32152,7 +32152,7 @@
       </c>
       <c r="K519" s="2" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>93</t>
         </is>
       </c>
       <c r="L519" s="2" t="inlineStr">
@@ -32209,7 +32209,7 @@
       </c>
       <c r="K520" s="2" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>23</t>
         </is>
       </c>
       <c r="L520" s="2" t="inlineStr">
@@ -32248,7 +32248,7 @@
         </is>
       </c>
       <c r="B521" s="3" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C521" s="3" t="inlineStr">
         <is>
@@ -32257,17 +32257,17 @@
       </c>
       <c r="D521" s="3" t="inlineStr">
         <is>
-          <t>Females per male, ages 15–64</t>
+          <t>Women per 100 Men (15–64)</t>
         </is>
       </c>
       <c r="E521" s="3" t="inlineStr">
         <is>
-          <t>Sex ratio ages 15–64, expressed as females per male (from World Factbook males-per-female via Wikipedia)</t>
+          <t>Sex ratio ages 15–64, women per 100 men (from World Factbook males-per-female via Wikipedia; = 100 ÷ Factbook ratio)</t>
         </is>
       </c>
       <c r="F521" s="3" t="inlineStr">
         <is>
-          <t>females per male</t>
+          <t>women per 100 men</t>
         </is>
       </c>
       <c r="G521" s="3" t="inlineStr">
@@ -32292,7 +32292,7 @@
       </c>
       <c r="K521" s="3" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>109</t>
         </is>
       </c>
       <c r="L521" s="3" t="inlineStr">
@@ -32312,7 +32312,7 @@
       </c>
       <c r="O521" s="3" t="inlineStr">
         <is>
-          <t>World Factbook male-to-female ratios for ages 15–64, via Wikipedia (rev 1372609821). Ranked as females per male (1 ÷ Factbook ratio). Qatar and similar Gulf states have many more men because of migrant labour. Caveat: Factbook estimates; national censuses can differ.</t>
+          <t>World Factbook male-to-female ratios for ages 15–64, via Wikipedia (rev 1372609821). Ranked as women per 100 men (100 ÷ Factbook males-per-female ratio). Qatar and similar Gulf states have many more men because of migrant labour. Caveat: Factbook estimates; national censuses can differ.</t>
         </is>
       </c>
       <c r="P521" s="3" t="inlineStr">
@@ -32343,7 +32343,7 @@
       </c>
       <c r="V521" s="3" t="inlineStr">
         <is>
-          <t>Females per Male (15–64)</t>
+          <t>Women per 100 Men (15–64)</t>
         </is>
       </c>
       <c r="W521" s="3" t="inlineStr">
@@ -32377,7 +32377,7 @@
       </c>
       <c r="K522" s="3" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>102</t>
         </is>
       </c>
       <c r="L522" s="3" t="inlineStr">
@@ -32434,7 +32434,7 @@
       </c>
       <c r="K523" s="3" t="inlineStr">
         <is>
-          <t>0.98</t>
+          <t>98</t>
         </is>
       </c>
       <c r="L523" s="3" t="inlineStr">
@@ -32491,7 +32491,7 @@
       </c>
       <c r="K524" s="3" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>94</t>
         </is>
       </c>
       <c r="L524" s="3" t="inlineStr">
@@ -32548,7 +32548,7 @@
       </c>
       <c r="K525" s="3" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>93</t>
         </is>
       </c>
       <c r="L525" s="3" t="inlineStr">
@@ -32605,7 +32605,7 @@
       </c>
       <c r="K526" s="3" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>70</t>
         </is>
       </c>
       <c r="L526" s="3" t="inlineStr">
@@ -32644,7 +32644,7 @@
         </is>
       </c>
       <c r="B527" s="2" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C527" s="2" t="inlineStr">
         <is>
@@ -32653,17 +32653,17 @@
       </c>
       <c r="D527" s="2" t="inlineStr">
         <is>
-          <t>Females per Male (65+)</t>
+          <t>Women per 100 Men (65+)</t>
         </is>
       </c>
       <c r="E527" s="2" t="inlineStr">
         <is>
-          <t>Sex ratio ages 65+, expressed as females per male (from World Factbook males-per-female via Wikipedia)</t>
+          <t>Sex ratio ages 65+, women per 100 men (from World Factbook males-per-female via Wikipedia; = 100 ÷ Factbook ratio)</t>
         </is>
       </c>
       <c r="F527" s="2" t="inlineStr">
         <is>
-          <t>females per male</t>
+          <t>women per 100 men</t>
         </is>
       </c>
       <c r="G527" s="2" t="inlineStr">
@@ -32688,7 +32688,7 @@
       </c>
       <c r="K527" s="2" t="inlineStr">
         <is>
-          <t>1.89</t>
+          <t>189</t>
         </is>
       </c>
       <c r="L527" s="2" t="inlineStr">
@@ -32708,7 +32708,7 @@
       </c>
       <c r="O527" s="2" t="inlineStr">
         <is>
-          <t>World Factbook male-to-female ratios for ages 65+, via Wikipedia (rev 1372609821). Ranked as females per male. Most countries have more older women than older men; the Gulf is an exception where working-age male migration still shapes the older cohorts. Caveat: Factbook estimates.</t>
+          <t>World Factbook male-to-female ratios for ages 65+, via Wikipedia (rev 1372609821). Ranked as women per 100 men. Most countries have more older women than older men; the Gulf is an exception where working-age male migration still shapes the older cohorts. Caveat: Factbook estimates.</t>
         </is>
       </c>
       <c r="P527" s="2" t="inlineStr">
@@ -32769,7 +32769,7 @@
       </c>
       <c r="K528" s="2" t="inlineStr">
         <is>
-          <t>1.82</t>
+          <t>182</t>
         </is>
       </c>
       <c r="L528" s="2" t="inlineStr">
@@ -32826,7 +32826,7 @@
       </c>
       <c r="K529" s="2" t="inlineStr">
         <is>
-          <t>1.69</t>
+          <t>169</t>
         </is>
       </c>
       <c r="L529" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="K530" s="2" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>152</t>
         </is>
       </c>
       <c r="L530" s="2" t="inlineStr">
@@ -32940,7 +32940,7 @@
       </c>
       <c r="K531" s="2" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>123</t>
         </is>
       </c>
       <c r="L531" s="2" t="inlineStr">
@@ -32997,7 +32997,7 @@
       </c>
       <c r="K532" s="2" t="inlineStr">
         <is>
-          <t>0.31</t>
+          <t>31</t>
         </is>
       </c>
       <c r="L532" s="2" t="inlineStr">
@@ -33029,8 +33029,1592 @@
       <c r="V532" s="2" t="inlineStr"/>
       <c r="W532" s="2" t="inlineStr"/>
     </row>
+    <row r="533">
+      <c r="A533" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-legal</t>
+        </is>
+      </c>
+      <c r="B533" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="C533" s="3" t="inlineStr">
+        <is>
+          <t>🏳️‍🌈</t>
+        </is>
+      </c>
+      <c r="D533" s="3" t="inlineStr">
+        <is>
+          <t>LGBT Legal Index</t>
+        </is>
+      </c>
+      <c r="E533" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex Legal Index (0–100; higher = better legal rights for LGBT people)</t>
+        </is>
+      </c>
+      <c r="F533" s="3" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G533" s="3" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H533" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I533" s="3" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="J533" s="3" t="inlineStr">
+        <is>
+          <t>🇫🇷</t>
+        </is>
+      </c>
+      <c r="K533" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="L533" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M533" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex Equality Index (Legal Index / Public Opinion Index)</t>
+        </is>
+      </c>
+      <c r="N533" s="3" t="inlineStr">
+        <is>
+          <t>https://www.equaldex.com/equality-index</t>
+        </is>
+      </c>
+      <c r="O533" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex Legal Index (0–100, higher = stronger legal LGBT rights), live chart on equaldex.com/equality-index (scraped 2026-10-23; Equaldex updates automatically as laws change). Afghanistan scores 0.</t>
+        </is>
+      </c>
+      <c r="P533" s="3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="Q533" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R533" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S533" s="3" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="T533" s="3" t="inlineStr"/>
+      <c r="U533" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-legal</t>
+        </is>
+      </c>
+      <c r="V533" s="3" t="inlineStr">
+        <is>
+          <t>LGBT Legal Index</t>
+        </is>
+      </c>
+      <c r="W533" s="3" t="inlineStr">
+        <is>
+          <t>Protect the Gays</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-legal</t>
+        </is>
+      </c>
+      <c r="B534" s="3" t="inlineStr"/>
+      <c r="C534" s="3" t="inlineStr"/>
+      <c r="D534" s="3" t="inlineStr"/>
+      <c r="E534" s="3" t="inlineStr"/>
+      <c r="F534" s="3" t="inlineStr"/>
+      <c r="G534" s="3" t="inlineStr"/>
+      <c r="H534" s="3" t="inlineStr"/>
+      <c r="I534" s="3" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="J534" s="3" t="inlineStr">
+        <is>
+          <t>🇹🇼</t>
+        </is>
+      </c>
+      <c r="K534" s="3" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="L534" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M534" s="3" t="inlineStr"/>
+      <c r="N534" s="3" t="inlineStr"/>
+      <c r="O534" s="3" t="inlineStr"/>
+      <c r="P534" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="Q534" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R534" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S534" s="3" t="inlineStr"/>
+      <c r="T534" s="3" t="inlineStr"/>
+      <c r="U534" s="3" t="inlineStr"/>
+      <c r="V534" s="3" t="inlineStr"/>
+      <c r="W534" s="3" t="inlineStr"/>
+    </row>
+    <row r="535">
+      <c r="A535" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-legal</t>
+        </is>
+      </c>
+      <c r="B535" s="3" t="inlineStr"/>
+      <c r="C535" s="3" t="inlineStr"/>
+      <c r="D535" s="3" t="inlineStr"/>
+      <c r="E535" s="3" t="inlineStr"/>
+      <c r="F535" s="3" t="inlineStr"/>
+      <c r="G535" s="3" t="inlineStr"/>
+      <c r="H535" s="3" t="inlineStr"/>
+      <c r="I535" s="3" t="inlineStr">
+        <is>
+          <t>Moldova</t>
+        </is>
+      </c>
+      <c r="J535" s="3" t="inlineStr">
+        <is>
+          <t>🇲🇩</t>
+        </is>
+      </c>
+      <c r="K535" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="L535" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M535" s="3" t="inlineStr"/>
+      <c r="N535" s="3" t="inlineStr"/>
+      <c r="O535" s="3" t="inlineStr"/>
+      <c r="P535" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="Q535" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R535" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S535" s="3" t="inlineStr"/>
+      <c r="T535" s="3" t="inlineStr"/>
+      <c r="U535" s="3" t="inlineStr"/>
+      <c r="V535" s="3" t="inlineStr"/>
+      <c r="W535" s="3" t="inlineStr"/>
+    </row>
+    <row r="536">
+      <c r="A536" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-legal</t>
+        </is>
+      </c>
+      <c r="B536" s="3" t="inlineStr"/>
+      <c r="C536" s="3" t="inlineStr"/>
+      <c r="D536" s="3" t="inlineStr"/>
+      <c r="E536" s="3" t="inlineStr"/>
+      <c r="F536" s="3" t="inlineStr"/>
+      <c r="G536" s="3" t="inlineStr"/>
+      <c r="H536" s="3" t="inlineStr"/>
+      <c r="I536" s="3" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="J536" s="3" t="inlineStr">
+        <is>
+          <t>🇰🇷</t>
+        </is>
+      </c>
+      <c r="K536" s="3" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="L536" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M536" s="3" t="inlineStr"/>
+      <c r="N536" s="3" t="inlineStr"/>
+      <c r="O536" s="3" t="inlineStr"/>
+      <c r="P536" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="Q536" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R536" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S536" s="3" t="inlineStr"/>
+      <c r="T536" s="3" t="inlineStr"/>
+      <c r="U536" s="3" t="inlineStr"/>
+      <c r="V536" s="3" t="inlineStr"/>
+      <c r="W536" s="3" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-legal</t>
+        </is>
+      </c>
+      <c r="B537" s="3" t="inlineStr"/>
+      <c r="C537" s="3" t="inlineStr"/>
+      <c r="D537" s="3" t="inlineStr"/>
+      <c r="E537" s="3" t="inlineStr"/>
+      <c r="F537" s="3" t="inlineStr"/>
+      <c r="G537" s="3" t="inlineStr"/>
+      <c r="H537" s="3" t="inlineStr"/>
+      <c r="I537" s="3" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="J537" s="3" t="inlineStr">
+        <is>
+          <t>🇷🇺</t>
+        </is>
+      </c>
+      <c r="K537" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="L537" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M537" s="3" t="inlineStr"/>
+      <c r="N537" s="3" t="inlineStr"/>
+      <c r="O537" s="3" t="inlineStr"/>
+      <c r="P537" s="3" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="Q537" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R537" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S537" s="3" t="inlineStr"/>
+      <c r="T537" s="3" t="inlineStr"/>
+      <c r="U537" s="3" t="inlineStr"/>
+      <c r="V537" s="3" t="inlineStr"/>
+      <c r="W537" s="3" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-legal</t>
+        </is>
+      </c>
+      <c r="B538" s="3" t="inlineStr"/>
+      <c r="C538" s="3" t="inlineStr"/>
+      <c r="D538" s="3" t="inlineStr"/>
+      <c r="E538" s="3" t="inlineStr"/>
+      <c r="F538" s="3" t="inlineStr"/>
+      <c r="G538" s="3" t="inlineStr"/>
+      <c r="H538" s="3" t="inlineStr"/>
+      <c r="I538" s="3" t="inlineStr">
+        <is>
+          <t>Afghanistan</t>
+        </is>
+      </c>
+      <c r="J538" s="3" t="inlineStr">
+        <is>
+          <t>🇦🇫</t>
+        </is>
+      </c>
+      <c r="K538" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L538" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M538" s="3" t="inlineStr"/>
+      <c r="N538" s="3" t="inlineStr"/>
+      <c r="O538" s="3" t="inlineStr"/>
+      <c r="P538" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="Q538" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R538" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S538" s="3" t="inlineStr"/>
+      <c r="T538" s="3" t="inlineStr"/>
+      <c r="U538" s="3" t="inlineStr"/>
+      <c r="V538" s="3" t="inlineStr"/>
+      <c r="W538" s="3" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-legal-b</t>
+        </is>
+      </c>
+      <c r="B539" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="C539" s="2" t="inlineStr">
+        <is>
+          <t>⚖️</t>
+        </is>
+      </c>
+      <c r="D539" s="2" t="inlineStr">
+        <is>
+          <t>LGBT Legal Index</t>
+        </is>
+      </c>
+      <c r="E539" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex Legal Index (0–100; higher = better legal rights for LGBT people)</t>
+        </is>
+      </c>
+      <c r="F539" s="2" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G539" s="2" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H539" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I539" s="2" t="inlineStr">
+        <is>
+          <t>Mongolia</t>
+        </is>
+      </c>
+      <c r="J539" s="2" t="inlineStr">
+        <is>
+          <t>🇲🇳</t>
+        </is>
+      </c>
+      <c r="K539" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="L539" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M539" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex Equality Index (Legal Index / Public Opinion Index)</t>
+        </is>
+      </c>
+      <c r="N539" s="2" t="inlineStr">
+        <is>
+          <t>https://www.equaldex.com/equality-index</t>
+        </is>
+      </c>
+      <c r="O539" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex Legal Index (0–100, higher = stronger legal LGBT rights), live chart on equaldex.com/equality-index (scraped 2026-10-23; Equaldex updates automatically as laws change). Afghanistan scores 0.</t>
+        </is>
+      </c>
+      <c r="P539" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="Q539" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R539" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S539" s="2" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="T539" s="2" t="inlineStr"/>
+      <c r="U539" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-legal</t>
+        </is>
+      </c>
+      <c r="V539" s="2" t="inlineStr">
+        <is>
+          <t>LGBT Legal Index</t>
+        </is>
+      </c>
+      <c r="W539" s="2" t="inlineStr">
+        <is>
+          <t>On the Books</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-legal-b</t>
+        </is>
+      </c>
+      <c r="B540" s="2" t="inlineStr"/>
+      <c r="C540" s="2" t="inlineStr"/>
+      <c r="D540" s="2" t="inlineStr"/>
+      <c r="E540" s="2" t="inlineStr"/>
+      <c r="F540" s="2" t="inlineStr"/>
+      <c r="G540" s="2" t="inlineStr"/>
+      <c r="H540" s="2" t="inlineStr"/>
+      <c r="I540" s="2" t="inlineStr">
+        <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="J540" s="2" t="inlineStr">
+        <is>
+          <t>🇺🇦</t>
+        </is>
+      </c>
+      <c r="K540" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="L540" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M540" s="2" t="inlineStr"/>
+      <c r="N540" s="2" t="inlineStr"/>
+      <c r="O540" s="2" t="inlineStr"/>
+      <c r="P540" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="Q540" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R540" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S540" s="2" t="inlineStr"/>
+      <c r="T540" s="2" t="inlineStr"/>
+      <c r="U540" s="2" t="inlineStr"/>
+      <c r="V540" s="2" t="inlineStr"/>
+      <c r="W540" s="2" t="inlineStr"/>
+    </row>
+    <row r="541">
+      <c r="A541" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-legal-b</t>
+        </is>
+      </c>
+      <c r="B541" s="2" t="inlineStr"/>
+      <c r="C541" s="2" t="inlineStr"/>
+      <c r="D541" s="2" t="inlineStr"/>
+      <c r="E541" s="2" t="inlineStr"/>
+      <c r="F541" s="2" t="inlineStr"/>
+      <c r="G541" s="2" t="inlineStr"/>
+      <c r="H541" s="2" t="inlineStr"/>
+      <c r="I541" s="2" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="J541" s="2" t="inlineStr">
+        <is>
+          <t>🇯🇵</t>
+        </is>
+      </c>
+      <c r="K541" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="L541" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M541" s="2" t="inlineStr"/>
+      <c r="N541" s="2" t="inlineStr"/>
+      <c r="O541" s="2" t="inlineStr"/>
+      <c r="P541" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="Q541" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R541" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S541" s="2" t="inlineStr"/>
+      <c r="T541" s="2" t="inlineStr"/>
+      <c r="U541" s="2" t="inlineStr"/>
+      <c r="V541" s="2" t="inlineStr"/>
+      <c r="W541" s="2" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-legal-b</t>
+        </is>
+      </c>
+      <c r="B542" s="2" t="inlineStr"/>
+      <c r="C542" s="2" t="inlineStr"/>
+      <c r="D542" s="2" t="inlineStr"/>
+      <c r="E542" s="2" t="inlineStr"/>
+      <c r="F542" s="2" t="inlineStr"/>
+      <c r="G542" s="2" t="inlineStr"/>
+      <c r="H542" s="2" t="inlineStr"/>
+      <c r="I542" s="2" t="inlineStr">
+        <is>
+          <t>Palestine</t>
+        </is>
+      </c>
+      <c r="J542" s="2" t="inlineStr">
+        <is>
+          <t>🇵🇸</t>
+        </is>
+      </c>
+      <c r="K542" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="L542" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M542" s="2" t="inlineStr"/>
+      <c r="N542" s="2" t="inlineStr"/>
+      <c r="O542" s="2" t="inlineStr"/>
+      <c r="P542" s="2" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="Q542" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R542" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S542" s="2" t="inlineStr"/>
+      <c r="T542" s="2" t="inlineStr"/>
+      <c r="U542" s="2" t="inlineStr"/>
+      <c r="V542" s="2" t="inlineStr"/>
+      <c r="W542" s="2" t="inlineStr"/>
+    </row>
+    <row r="543">
+      <c r="A543" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-legal-b</t>
+        </is>
+      </c>
+      <c r="B543" s="2" t="inlineStr"/>
+      <c r="C543" s="2" t="inlineStr"/>
+      <c r="D543" s="2" t="inlineStr"/>
+      <c r="E543" s="2" t="inlineStr"/>
+      <c r="F543" s="2" t="inlineStr"/>
+      <c r="G543" s="2" t="inlineStr"/>
+      <c r="H543" s="2" t="inlineStr"/>
+      <c r="I543" s="2" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="J543" s="2" t="inlineStr">
+        <is>
+          <t>🇮🇩</t>
+        </is>
+      </c>
+      <c r="K543" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="L543" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M543" s="2" t="inlineStr"/>
+      <c r="N543" s="2" t="inlineStr"/>
+      <c r="O543" s="2" t="inlineStr"/>
+      <c r="P543" s="2" t="inlineStr">
+        <is>
+          <t>149</t>
+        </is>
+      </c>
+      <c r="Q543" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R543" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S543" s="2" t="inlineStr"/>
+      <c r="T543" s="2" t="inlineStr"/>
+      <c r="U543" s="2" t="inlineStr"/>
+      <c r="V543" s="2" t="inlineStr"/>
+      <c r="W543" s="2" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-legal-b</t>
+        </is>
+      </c>
+      <c r="B544" s="2" t="inlineStr"/>
+      <c r="C544" s="2" t="inlineStr"/>
+      <c r="D544" s="2" t="inlineStr"/>
+      <c r="E544" s="2" t="inlineStr"/>
+      <c r="F544" s="2" t="inlineStr"/>
+      <c r="G544" s="2" t="inlineStr"/>
+      <c r="H544" s="2" t="inlineStr"/>
+      <c r="I544" s="2" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J544" s="2" t="inlineStr">
+        <is>
+          <t>🇳🇬</t>
+        </is>
+      </c>
+      <c r="K544" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="L544" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M544" s="2" t="inlineStr"/>
+      <c r="N544" s="2" t="inlineStr"/>
+      <c r="O544" s="2" t="inlineStr"/>
+      <c r="P544" s="2" t="inlineStr">
+        <is>
+          <t>163</t>
+        </is>
+      </c>
+      <c r="Q544" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R544" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S544" s="2" t="inlineStr"/>
+      <c r="T544" s="2" t="inlineStr"/>
+      <c r="U544" s="2" t="inlineStr"/>
+      <c r="V544" s="2" t="inlineStr"/>
+      <c r="W544" s="2" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-opinion</t>
+        </is>
+      </c>
+      <c r="B545" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="C545" s="3" t="inlineStr">
+        <is>
+          <t>💬</t>
+        </is>
+      </c>
+      <c r="D545" s="3" t="inlineStr">
+        <is>
+          <t>LGBT Public Opinion Index</t>
+        </is>
+      </c>
+      <c r="E545" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex Public Opinion Index (0–100; higher = more accepting public attitudes)</t>
+        </is>
+      </c>
+      <c r="F545" s="3" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G545" s="3" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H545" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I545" s="3" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="J545" s="3" t="inlineStr">
+        <is>
+          <t>🇳🇴</t>
+        </is>
+      </c>
+      <c r="K545" s="3" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="L545" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M545" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex Equality Index (Legal Index / Public Opinion Index)</t>
+        </is>
+      </c>
+      <c r="N545" s="3" t="inlineStr">
+        <is>
+          <t>https://www.equaldex.com/equality-index</t>
+        </is>
+      </c>
+      <c r="O545" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex Public Opinion Index (0–100, higher = more accepting public attitudes), live chart on equaldex.com/equality-index (scraped 2026-10-23; Equaldex updates automatically).</t>
+        </is>
+      </c>
+      <c r="P545" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q545" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R545" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S545" s="3" t="inlineStr">
+        <is>
+          <t>heart</t>
+        </is>
+      </c>
+      <c r="T545" s="3" t="inlineStr"/>
+      <c r="U545" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-opinion</t>
+        </is>
+      </c>
+      <c r="V545" s="3" t="inlineStr">
+        <is>
+          <t>LGBT Public Opinion Index</t>
+        </is>
+      </c>
+      <c r="W545" s="3" t="inlineStr">
+        <is>
+          <t>Why are you gay?</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-opinion</t>
+        </is>
+      </c>
+      <c r="B546" s="3" t="inlineStr"/>
+      <c r="C546" s="3" t="inlineStr"/>
+      <c r="D546" s="3" t="inlineStr"/>
+      <c r="E546" s="3" t="inlineStr"/>
+      <c r="F546" s="3" t="inlineStr"/>
+      <c r="G546" s="3" t="inlineStr"/>
+      <c r="H546" s="3" t="inlineStr"/>
+      <c r="I546" s="3" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="J546" s="3" t="inlineStr">
+        <is>
+          <t>🇹🇭</t>
+        </is>
+      </c>
+      <c r="K546" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="L546" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M546" s="3" t="inlineStr"/>
+      <c r="N546" s="3" t="inlineStr"/>
+      <c r="O546" s="3" t="inlineStr"/>
+      <c r="P546" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="Q546" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R546" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S546" s="3" t="inlineStr"/>
+      <c r="T546" s="3" t="inlineStr"/>
+      <c r="U546" s="3" t="inlineStr"/>
+      <c r="V546" s="3" t="inlineStr"/>
+      <c r="W546" s="3" t="inlineStr"/>
+    </row>
+    <row r="547">
+      <c r="A547" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-opinion</t>
+        </is>
+      </c>
+      <c r="B547" s="3" t="inlineStr"/>
+      <c r="C547" s="3" t="inlineStr"/>
+      <c r="D547" s="3" t="inlineStr"/>
+      <c r="E547" s="3" t="inlineStr"/>
+      <c r="F547" s="3" t="inlineStr"/>
+      <c r="G547" s="3" t="inlineStr"/>
+      <c r="H547" s="3" t="inlineStr"/>
+      <c r="I547" s="3" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="J547" s="3" t="inlineStr">
+        <is>
+          <t>🇨🇳</t>
+        </is>
+      </c>
+      <c r="K547" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="L547" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M547" s="3" t="inlineStr"/>
+      <c r="N547" s="3" t="inlineStr"/>
+      <c r="O547" s="3" t="inlineStr"/>
+      <c r="P547" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="Q547" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R547" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S547" s="3" t="inlineStr"/>
+      <c r="T547" s="3" t="inlineStr"/>
+      <c r="U547" s="3" t="inlineStr"/>
+      <c r="V547" s="3" t="inlineStr"/>
+      <c r="W547" s="3" t="inlineStr"/>
+    </row>
+    <row r="548">
+      <c r="A548" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-opinion</t>
+        </is>
+      </c>
+      <c r="B548" s="3" t="inlineStr"/>
+      <c r="C548" s="3" t="inlineStr"/>
+      <c r="D548" s="3" t="inlineStr"/>
+      <c r="E548" s="3" t="inlineStr"/>
+      <c r="F548" s="3" t="inlineStr"/>
+      <c r="G548" s="3" t="inlineStr"/>
+      <c r="H548" s="3" t="inlineStr"/>
+      <c r="I548" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="J548" s="3" t="inlineStr">
+        <is>
+          <t>🇺🇸</t>
+        </is>
+      </c>
+      <c r="K548" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="L548" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M548" s="3" t="inlineStr"/>
+      <c r="N548" s="3" t="inlineStr"/>
+      <c r="O548" s="3" t="inlineStr"/>
+      <c r="P548" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="Q548" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R548" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S548" s="3" t="inlineStr"/>
+      <c r="T548" s="3" t="inlineStr"/>
+      <c r="U548" s="3" t="inlineStr"/>
+      <c r="V548" s="3" t="inlineStr"/>
+      <c r="W548" s="3" t="inlineStr"/>
+    </row>
+    <row r="549">
+      <c r="A549" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-opinion</t>
+        </is>
+      </c>
+      <c r="B549" s="3" t="inlineStr"/>
+      <c r="C549" s="3" t="inlineStr"/>
+      <c r="D549" s="3" t="inlineStr"/>
+      <c r="E549" s="3" t="inlineStr"/>
+      <c r="F549" s="3" t="inlineStr"/>
+      <c r="G549" s="3" t="inlineStr"/>
+      <c r="H549" s="3" t="inlineStr"/>
+      <c r="I549" s="3" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="J549" s="3" t="inlineStr">
+        <is>
+          <t>🇮🇱</t>
+        </is>
+      </c>
+      <c r="K549" s="3" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="L549" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M549" s="3" t="inlineStr"/>
+      <c r="N549" s="3" t="inlineStr"/>
+      <c r="O549" s="3" t="inlineStr"/>
+      <c r="P549" s="3" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="Q549" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R549" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S549" s="3" t="inlineStr"/>
+      <c r="T549" s="3" t="inlineStr"/>
+      <c r="U549" s="3" t="inlineStr"/>
+      <c r="V549" s="3" t="inlineStr"/>
+      <c r="W549" s="3" t="inlineStr"/>
+    </row>
+    <row r="550">
+      <c r="A550" s="3" t="inlineStr">
+        <is>
+          <t>equaldex-opinion</t>
+        </is>
+      </c>
+      <c r="B550" s="3" t="inlineStr"/>
+      <c r="C550" s="3" t="inlineStr"/>
+      <c r="D550" s="3" t="inlineStr"/>
+      <c r="E550" s="3" t="inlineStr"/>
+      <c r="F550" s="3" t="inlineStr"/>
+      <c r="G550" s="3" t="inlineStr"/>
+      <c r="H550" s="3" t="inlineStr"/>
+      <c r="I550" s="3" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="J550" s="3" t="inlineStr">
+        <is>
+          <t>🇺🇬</t>
+        </is>
+      </c>
+      <c r="K550" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="L550" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M550" s="3" t="inlineStr"/>
+      <c r="N550" s="3" t="inlineStr"/>
+      <c r="O550" s="3" t="inlineStr"/>
+      <c r="P550" s="3" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="Q550" s="3" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R550" s="3" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S550" s="3" t="inlineStr"/>
+      <c r="T550" s="3" t="inlineStr"/>
+      <c r="U550" s="3" t="inlineStr"/>
+      <c r="V550" s="3" t="inlineStr"/>
+      <c r="W550" s="3" t="inlineStr"/>
+    </row>
+    <row r="551">
+      <c r="A551" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-opinion-b</t>
+        </is>
+      </c>
+      <c r="B551" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="C551" s="2" t="inlineStr">
+        <is>
+          <t>🗳️</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>LGBT Public Opinion Index</t>
+        </is>
+      </c>
+      <c r="E551" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex Public Opinion Index (0–100; higher = more accepting public attitudes)</t>
+        </is>
+      </c>
+      <c r="F551" s="2" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="G551" s="2" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H551" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I551" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J551" s="2" t="inlineStr">
+        <is>
+          <t>🇮🇳</t>
+        </is>
+      </c>
+      <c r="K551" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="L551" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M551" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex Equality Index (Legal Index / Public Opinion Index)</t>
+        </is>
+      </c>
+      <c r="N551" s="2" t="inlineStr">
+        <is>
+          <t>https://www.equaldex.com/equality-index</t>
+        </is>
+      </c>
+      <c r="O551" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex Public Opinion Index (0–100, higher = more accepting public attitudes), live chart on equaldex.com/equality-index (scraped 2026-10-23; Equaldex updates automatically).</t>
+        </is>
+      </c>
+      <c r="P551" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="Q551" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R551" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S551" s="2" t="inlineStr">
+        <is>
+          <t>heart</t>
+        </is>
+      </c>
+      <c r="T551" s="2" t="inlineStr"/>
+      <c r="U551" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-opinion</t>
+        </is>
+      </c>
+      <c r="V551" s="2" t="inlineStr">
+        <is>
+          <t>LGBT Public Opinion Index</t>
+        </is>
+      </c>
+      <c r="W551" s="2" t="inlineStr">
+        <is>
+          <t>Asking for a Friend</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-opinion-b</t>
+        </is>
+      </c>
+      <c r="B552" s="2" t="inlineStr"/>
+      <c r="C552" s="2" t="inlineStr"/>
+      <c r="D552" s="2" t="inlineStr"/>
+      <c r="E552" s="2" t="inlineStr"/>
+      <c r="F552" s="2" t="inlineStr"/>
+      <c r="G552" s="2" t="inlineStr"/>
+      <c r="H552" s="2" t="inlineStr"/>
+      <c r="I552" s="2" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="J552" s="2" t="inlineStr">
+        <is>
+          <t>🇰🇷</t>
+        </is>
+      </c>
+      <c r="K552" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="L552" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M552" s="2" t="inlineStr"/>
+      <c r="N552" s="2" t="inlineStr"/>
+      <c r="O552" s="2" t="inlineStr"/>
+      <c r="P552" s="2" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="Q552" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R552" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S552" s="2" t="inlineStr"/>
+      <c r="T552" s="2" t="inlineStr"/>
+      <c r="U552" s="2" t="inlineStr"/>
+      <c r="V552" s="2" t="inlineStr"/>
+      <c r="W552" s="2" t="inlineStr"/>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-opinion-b</t>
+        </is>
+      </c>
+      <c r="B553" s="2" t="inlineStr"/>
+      <c r="C553" s="2" t="inlineStr"/>
+      <c r="D553" s="2" t="inlineStr"/>
+      <c r="E553" s="2" t="inlineStr"/>
+      <c r="F553" s="2" t="inlineStr"/>
+      <c r="G553" s="2" t="inlineStr"/>
+      <c r="H553" s="2" t="inlineStr"/>
+      <c r="I553" s="2" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="J553" s="2" t="inlineStr">
+        <is>
+          <t>🇵🇰</t>
+        </is>
+      </c>
+      <c r="K553" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="L553" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M553" s="2" t="inlineStr"/>
+      <c r="N553" s="2" t="inlineStr"/>
+      <c r="O553" s="2" t="inlineStr"/>
+      <c r="P553" s="2" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="Q553" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R553" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S553" s="2" t="inlineStr"/>
+      <c r="T553" s="2" t="inlineStr"/>
+      <c r="U553" s="2" t="inlineStr"/>
+      <c r="V553" s="2" t="inlineStr"/>
+      <c r="W553" s="2" t="inlineStr"/>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-opinion-b</t>
+        </is>
+      </c>
+      <c r="B554" s="2" t="inlineStr"/>
+      <c r="C554" s="2" t="inlineStr"/>
+      <c r="D554" s="2" t="inlineStr"/>
+      <c r="E554" s="2" t="inlineStr"/>
+      <c r="F554" s="2" t="inlineStr"/>
+      <c r="G554" s="2" t="inlineStr"/>
+      <c r="H554" s="2" t="inlineStr"/>
+      <c r="I554" s="2" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="J554" s="2" t="inlineStr">
+        <is>
+          <t>🇷🇺</t>
+        </is>
+      </c>
+      <c r="K554" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="L554" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M554" s="2" t="inlineStr"/>
+      <c r="N554" s="2" t="inlineStr"/>
+      <c r="O554" s="2" t="inlineStr"/>
+      <c r="P554" s="2" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="Q554" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R554" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S554" s="2" t="inlineStr"/>
+      <c r="T554" s="2" t="inlineStr"/>
+      <c r="U554" s="2" t="inlineStr"/>
+      <c r="V554" s="2" t="inlineStr"/>
+      <c r="W554" s="2" t="inlineStr"/>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-opinion-b</t>
+        </is>
+      </c>
+      <c r="B555" s="2" t="inlineStr"/>
+      <c r="C555" s="2" t="inlineStr"/>
+      <c r="D555" s="2" t="inlineStr"/>
+      <c r="E555" s="2" t="inlineStr"/>
+      <c r="F555" s="2" t="inlineStr"/>
+      <c r="G555" s="2" t="inlineStr"/>
+      <c r="H555" s="2" t="inlineStr"/>
+      <c r="I555" s="2" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="J555" s="2" t="inlineStr">
+        <is>
+          <t>🇺🇬</t>
+        </is>
+      </c>
+      <c r="K555" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="L555" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M555" s="2" t="inlineStr"/>
+      <c r="N555" s="2" t="inlineStr"/>
+      <c r="O555" s="2" t="inlineStr"/>
+      <c r="P555" s="2" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="Q555" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R555" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S555" s="2" t="inlineStr"/>
+      <c r="T555" s="2" t="inlineStr"/>
+      <c r="U555" s="2" t="inlineStr"/>
+      <c r="V555" s="2" t="inlineStr"/>
+      <c r="W555" s="2" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>equaldex-opinion-b</t>
+        </is>
+      </c>
+      <c r="B556" s="2" t="inlineStr"/>
+      <c r="C556" s="2" t="inlineStr"/>
+      <c r="D556" s="2" t="inlineStr"/>
+      <c r="E556" s="2" t="inlineStr"/>
+      <c r="F556" s="2" t="inlineStr"/>
+      <c r="G556" s="2" t="inlineStr"/>
+      <c r="H556" s="2" t="inlineStr"/>
+      <c r="I556" s="2" t="inlineStr">
+        <is>
+          <t>Afghanistan</t>
+        </is>
+      </c>
+      <c r="J556" s="2" t="inlineStr">
+        <is>
+          <t>🇦🇫</t>
+        </is>
+      </c>
+      <c r="K556" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L556" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex live (scraped 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="M556" s="2" t="inlineStr"/>
+      <c r="N556" s="2" t="inlineStr"/>
+      <c r="O556" s="2" t="inlineStr"/>
+      <c r="P556" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="Q556" s="2" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="R556" s="2" t="inlineStr">
+        <is>
+          <t>Equaldex countries</t>
+        </is>
+      </c>
+      <c r="S556" s="2" t="inlineStr"/>
+      <c r="T556" s="2" t="inlineStr"/>
+      <c r="U556" s="2" t="inlineStr"/>
+      <c r="V556" s="2" t="inlineStr"/>
+      <c r="W556" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W532"/>
+  <autoFilter ref="A1:W556"/>
   <dataValidations count="2">
     <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"top,bottom"</formula1>
@@ -80872,7 +82456,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -81085,7 +82669,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -81156,7 +82740,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -81594,7 +83178,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -81899,7 +83483,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -82267,7 +83851,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
v12.2: Tier it + Pew meaning Match/Tier + Devil's Dice gambling Rank its
New Tier it mode (God is Meaningful — Pew 2021 religion mentions).
What Matters Most Match it (Pew meaning-of-life cross-country).
Devil's Dice / Snake Eyes from Pew Spring 2025 gambling morality.
Rank it scores tied values by slot value. Schedule 124.
</commit_message>
<xml_diff>
--- a/puzzles.xlsx
+++ b/puzzles.xlsx
@@ -13,15 +13,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hint_bank" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top5_puzzles" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="match_puzzles" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOW TO EDIT" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tier_puzzles" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOW TO EDIT" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'puzzles'!$A$1:$W$556</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'puzzles'!$A$1:$W$568</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'country_lists'!$A$1:$G$1009</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'country_info'!$A$1:$L$222</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'hint_bank'!$A$1:$H$181</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'top5_puzzles'!$A$1:$O$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'match_puzzles'!$A$1:$Q$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'match_puzzles'!$A$1:$Q$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'tier_puzzles'!$A$1:$U$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W556"/>
+  <dimension ref="A1:W568"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4443,7 +4445,7 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
@@ -4754,7 +4756,7 @@
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
@@ -5376,7 +5378,7 @@
         </is>
       </c>
       <c r="B85" s="3" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
@@ -5868,7 +5870,7 @@
         </is>
       </c>
       <c r="B93" s="3" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
@@ -6530,7 +6532,7 @@
         </is>
       </c>
       <c r="B103" s="3" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
@@ -7072,7 +7074,7 @@
         </is>
       </c>
       <c r="B113" s="3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
@@ -7569,7 +7571,7 @@
         </is>
       </c>
       <c r="B122" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
@@ -7795,7 +7797,7 @@
         </is>
       </c>
       <c r="B126" s="2" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
@@ -8021,7 +8023,7 @@
         </is>
       </c>
       <c r="B130" s="3" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
@@ -8247,7 +8249,7 @@
         </is>
       </c>
       <c r="B134" s="2" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
@@ -8578,7 +8580,7 @@
         </is>
       </c>
       <c r="B139" s="3" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
@@ -8849,7 +8851,7 @@
         </is>
       </c>
       <c r="B144" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
@@ -9180,7 +9182,7 @@
         </is>
       </c>
       <c r="B149" s="3" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
@@ -9451,7 +9453,7 @@
         </is>
       </c>
       <c r="B154" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
@@ -10655,7 +10657,7 @@
         </is>
       </c>
       <c r="B174" s="2" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
@@ -10978,7 +10980,7 @@
         </is>
       </c>
       <c r="B179" s="3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
@@ -11289,7 +11291,7 @@
         </is>
       </c>
       <c r="B184" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
@@ -11911,7 +11913,7 @@
         </is>
       </c>
       <c r="B194" s="2" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
@@ -12230,7 +12232,7 @@
         </is>
       </c>
       <c r="B199" s="3" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
@@ -12868,7 +12870,7 @@
         </is>
       </c>
       <c r="B209" s="3" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
@@ -13179,7 +13181,7 @@
         </is>
       </c>
       <c r="B214" s="2" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
@@ -13490,7 +13492,7 @@
         </is>
       </c>
       <c r="B219" s="3" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
@@ -13817,7 +13819,7 @@
         </is>
       </c>
       <c r="B224" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
@@ -14156,7 +14158,7 @@
         </is>
       </c>
       <c r="B229" s="3" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
@@ -14487,7 +14489,7 @@
         </is>
       </c>
       <c r="B234" s="2" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
@@ -14798,7 +14800,7 @@
         </is>
       </c>
       <c r="B239" s="3" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
@@ -15109,7 +15111,7 @@
         </is>
       </c>
       <c r="B244" s="2" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
@@ -15428,7 +15430,7 @@
         </is>
       </c>
       <c r="B249" s="3" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
@@ -15800,7 +15802,7 @@
         </is>
       </c>
       <c r="B255" s="2" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
@@ -16099,7 +16101,7 @@
         </is>
       </c>
       <c r="B260" s="3" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
@@ -16746,7 +16748,7 @@
         </is>
       </c>
       <c r="B271" s="3" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
@@ -17041,7 +17043,7 @@
         </is>
       </c>
       <c r="B276" s="2" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
@@ -17340,7 +17342,7 @@
         </is>
       </c>
       <c r="B281" s="3" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
@@ -17639,7 +17641,7 @@
         </is>
       </c>
       <c r="B286" s="2" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
@@ -17958,7 +17960,7 @@
         </is>
       </c>
       <c r="B291" s="3" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
@@ -18330,7 +18332,7 @@
         </is>
       </c>
       <c r="B297" s="2" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
@@ -18629,7 +18631,7 @@
         </is>
       </c>
       <c r="B302" s="3" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C302" s="3" t="inlineStr">
         <is>
@@ -18928,7 +18930,7 @@
         </is>
       </c>
       <c r="B307" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
@@ -19272,7 +19274,7 @@
         </is>
       </c>
       <c r="B313" s="3" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C313" s="3" t="inlineStr">
         <is>
@@ -19567,7 +19569,7 @@
         </is>
       </c>
       <c r="B318" s="2" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
@@ -19866,7 +19868,7 @@
         </is>
       </c>
       <c r="B323" s="3" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C323" s="3" t="inlineStr">
         <is>
@@ -20165,7 +20167,7 @@
         </is>
       </c>
       <c r="B328" s="2" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
@@ -20464,7 +20466,7 @@
         </is>
       </c>
       <c r="B333" s="3" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C333" s="3" t="inlineStr">
         <is>
@@ -20759,7 +20761,7 @@
         </is>
       </c>
       <c r="B338" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
@@ -21054,7 +21056,7 @@
         </is>
       </c>
       <c r="B343" s="3" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C343" s="3" t="inlineStr">
         <is>
@@ -21701,7 +21703,7 @@
         </is>
       </c>
       <c r="B354" s="3" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C354" s="3" t="inlineStr">
         <is>
@@ -22000,7 +22002,7 @@
         </is>
       </c>
       <c r="B359" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
@@ -22299,7 +22301,7 @@
         </is>
       </c>
       <c r="B364" s="3" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C364" s="3" t="inlineStr">
         <is>
@@ -22594,7 +22596,7 @@
         </is>
       </c>
       <c r="B369" s="2" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
@@ -22889,7 +22891,7 @@
         </is>
       </c>
       <c r="B374" s="3" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
@@ -23188,7 +23190,7 @@
         </is>
       </c>
       <c r="B379" s="2" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
@@ -23487,7 +23489,7 @@
         </is>
       </c>
       <c r="B384" s="3" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C384" s="3" t="inlineStr">
         <is>
@@ -23806,7 +23808,7 @@
         </is>
       </c>
       <c r="B389" s="2" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
@@ -24105,7 +24107,7 @@
         </is>
       </c>
       <c r="B394" s="3" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C394" s="3" t="inlineStr">
         <is>
@@ -24436,7 +24438,7 @@
         </is>
       </c>
       <c r="B399" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
@@ -24767,7 +24769,7 @@
         </is>
       </c>
       <c r="B404" s="3" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C404" s="3" t="inlineStr">
         <is>
@@ -25874,7 +25876,7 @@
         </is>
       </c>
       <c r="B421" s="2" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
@@ -26205,7 +26207,7 @@
         </is>
       </c>
       <c r="B426" s="3" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C426" s="3" t="inlineStr">
         <is>
@@ -26536,7 +26538,7 @@
         </is>
       </c>
       <c r="B431" s="2" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
@@ -26867,7 +26869,7 @@
         </is>
       </c>
       <c r="B436" s="3" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C436" s="3" t="inlineStr">
         <is>
@@ -27198,7 +27200,7 @@
         </is>
       </c>
       <c r="B441" s="2" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
@@ -27472,7 +27474,7 @@
         </is>
       </c>
       <c r="B445" s="3" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C445" s="3" t="inlineStr">
         <is>
@@ -27746,7 +27748,7 @@
         </is>
       </c>
       <c r="B449" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
@@ -28020,7 +28022,7 @@
         </is>
       </c>
       <c r="B453" s="3" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C453" s="3" t="inlineStr">
         <is>
@@ -28412,7 +28414,7 @@
         </is>
       </c>
       <c r="B459" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C459" s="2" t="inlineStr">
         <is>
@@ -28804,7 +28806,7 @@
         </is>
       </c>
       <c r="B465" s="3" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C465" s="3" t="inlineStr">
         <is>
@@ -29103,7 +29105,7 @@
         </is>
       </c>
       <c r="B470" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C470" s="2" t="inlineStr">
         <is>
@@ -29451,7 +29453,7 @@
         </is>
       </c>
       <c r="B476" s="3" t="n">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C476" s="3" t="inlineStr">
         <is>
@@ -30187,7 +30189,7 @@
         </is>
       </c>
       <c r="B488" s="3" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C488" s="3" t="inlineStr">
         <is>
@@ -30555,7 +30557,7 @@
         </is>
       </c>
       <c r="B494" s="2" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
@@ -30826,7 +30828,7 @@
         </is>
       </c>
       <c r="B499" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C499" s="3" t="inlineStr">
         <is>
@@ -31100,7 +31102,7 @@
         </is>
       </c>
       <c r="B503" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
@@ -31488,7 +31490,7 @@
         </is>
       </c>
       <c r="B509" s="3" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C509" s="3" t="inlineStr">
         <is>
@@ -31852,7 +31854,7 @@
         </is>
       </c>
       <c r="B515" s="2" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C515" s="2" t="inlineStr">
         <is>
@@ -32248,7 +32250,7 @@
         </is>
       </c>
       <c r="B521" s="3" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C521" s="3" t="inlineStr">
         <is>
@@ -32644,7 +32646,7 @@
         </is>
       </c>
       <c r="B527" s="2" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C527" s="2" t="inlineStr">
         <is>
@@ -33036,7 +33038,7 @@
         </is>
       </c>
       <c r="B533" s="3" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C533" s="3" t="inlineStr">
         <is>
@@ -33432,7 +33434,7 @@
         </is>
       </c>
       <c r="B539" s="2" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C539" s="2" t="inlineStr">
         <is>
@@ -33828,7 +33830,7 @@
         </is>
       </c>
       <c r="B545" s="3" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C545" s="3" t="inlineStr">
         <is>
@@ -34224,7 +34226,7 @@
         </is>
       </c>
       <c r="B551" s="2" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C551" s="2" t="inlineStr">
         <is>
@@ -34613,8 +34615,656 @@
       <c r="V556" s="2" t="inlineStr"/>
       <c r="W556" s="2" t="inlineStr"/>
     </row>
+    <row r="557">
+      <c r="A557" s="3" t="inlineStr">
+        <is>
+          <t>gambling-immoral</t>
+        </is>
+      </c>
+      <c r="B557" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C557" s="3" t="inlineStr">
+        <is>
+          <t>🎲</t>
+        </is>
+      </c>
+      <c r="D557" s="3" t="inlineStr">
+        <is>
+          <t>% who say gambling is morally wrong</t>
+        </is>
+      </c>
+      <c r="E557" s="3" t="inlineStr">
+        <is>
+          <t>Gambling is morally unacceptable (US: morally wrong)</t>
+        </is>
+      </c>
+      <c r="F557" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G557" s="3" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H557" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I557" s="3" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="J557" s="3" t="inlineStr">
+        <is>
+          <t>🇮🇩</t>
+        </is>
+      </c>
+      <c r="K557" s="3" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="L557" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M557" s="3" t="inlineStr">
+        <is>
+          <t>Pew Research Center Spring 2025 Global Attitudes (Q17d gambling)</t>
+        </is>
+      </c>
+      <c r="N557" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pewresearch.org/short-reads/2026/03/16/americans-are-less-likely-than-people-in-many-other-countries-to-see-gambling-as-morally-wrong/</t>
+        </is>
+      </c>
+      <c r="O557" s="3" t="inlineStr">
+        <is>
+          <t>Indonesians (89%) are three times as likely as Americans (29%) to call gambling morally wrong — and half of Americans say it isn't a moral issue at all, more than any other public surveyed.</t>
+        </is>
+      </c>
+      <c r="P557" s="3" t="inlineStr"/>
+      <c r="Q557" s="3" t="inlineStr"/>
+      <c r="R557" s="3" t="inlineStr"/>
+      <c r="S557" s="3" t="inlineStr">
+        <is>
+          <t>sparkles</t>
+        </is>
+      </c>
+      <c r="T557" s="3" t="inlineStr"/>
+      <c r="U557" s="3" t="inlineStr">
+        <is>
+          <t>pew-gambling-immoral</t>
+        </is>
+      </c>
+      <c r="V557" s="3" t="inlineStr">
+        <is>
+          <t>Gambling Immoral</t>
+        </is>
+      </c>
+      <c r="W557" s="3" t="inlineStr">
+        <is>
+          <t>Devil's Dice</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="3" t="inlineStr">
+        <is>
+          <t>gambling-immoral</t>
+        </is>
+      </c>
+      <c r="B558" s="3" t="inlineStr"/>
+      <c r="C558" s="3" t="inlineStr"/>
+      <c r="D558" s="3" t="inlineStr"/>
+      <c r="E558" s="3" t="inlineStr"/>
+      <c r="F558" s="3" t="inlineStr"/>
+      <c r="G558" s="3" t="inlineStr"/>
+      <c r="H558" s="3" t="inlineStr"/>
+      <c r="I558" s="3" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="J558" s="3" t="inlineStr">
+        <is>
+          <t>🇰🇷</t>
+        </is>
+      </c>
+      <c r="K558" s="3" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="L558" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M558" s="3" t="inlineStr"/>
+      <c r="N558" s="3" t="inlineStr"/>
+      <c r="O558" s="3" t="inlineStr"/>
+      <c r="P558" s="3" t="inlineStr"/>
+      <c r="Q558" s="3" t="inlineStr"/>
+      <c r="R558" s="3" t="inlineStr"/>
+      <c r="S558" s="3" t="inlineStr"/>
+      <c r="T558" s="3" t="inlineStr"/>
+      <c r="U558" s="3" t="inlineStr"/>
+      <c r="V558" s="3" t="inlineStr"/>
+      <c r="W558" s="3" t="inlineStr"/>
+    </row>
+    <row r="559">
+      <c r="A559" s="3" t="inlineStr">
+        <is>
+          <t>gambling-immoral</t>
+        </is>
+      </c>
+      <c r="B559" s="3" t="inlineStr"/>
+      <c r="C559" s="3" t="inlineStr"/>
+      <c r="D559" s="3" t="inlineStr"/>
+      <c r="E559" s="3" t="inlineStr"/>
+      <c r="F559" s="3" t="inlineStr"/>
+      <c r="G559" s="3" t="inlineStr"/>
+      <c r="H559" s="3" t="inlineStr"/>
+      <c r="I559" s="3" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="J559" s="3" t="inlineStr">
+        <is>
+          <t>🇮🇱</t>
+        </is>
+      </c>
+      <c r="K559" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="L559" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M559" s="3" t="inlineStr"/>
+      <c r="N559" s="3" t="inlineStr"/>
+      <c r="O559" s="3" t="inlineStr"/>
+      <c r="P559" s="3" t="inlineStr"/>
+      <c r="Q559" s="3" t="inlineStr"/>
+      <c r="R559" s="3" t="inlineStr"/>
+      <c r="S559" s="3" t="inlineStr"/>
+      <c r="T559" s="3" t="inlineStr"/>
+      <c r="U559" s="3" t="inlineStr"/>
+      <c r="V559" s="3" t="inlineStr"/>
+      <c r="W559" s="3" t="inlineStr"/>
+    </row>
+    <row r="560">
+      <c r="A560" s="3" t="inlineStr">
+        <is>
+          <t>gambling-immoral</t>
+        </is>
+      </c>
+      <c r="B560" s="3" t="inlineStr"/>
+      <c r="C560" s="3" t="inlineStr"/>
+      <c r="D560" s="3" t="inlineStr"/>
+      <c r="E560" s="3" t="inlineStr"/>
+      <c r="F560" s="3" t="inlineStr"/>
+      <c r="G560" s="3" t="inlineStr"/>
+      <c r="H560" s="3" t="inlineStr"/>
+      <c r="I560" s="3" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="J560" s="3" t="inlineStr">
+        <is>
+          <t>🇲🇽</t>
+        </is>
+      </c>
+      <c r="K560" s="3" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="L560" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M560" s="3" t="inlineStr"/>
+      <c r="N560" s="3" t="inlineStr"/>
+      <c r="O560" s="3" t="inlineStr"/>
+      <c r="P560" s="3" t="inlineStr"/>
+      <c r="Q560" s="3" t="inlineStr"/>
+      <c r="R560" s="3" t="inlineStr"/>
+      <c r="S560" s="3" t="inlineStr"/>
+      <c r="T560" s="3" t="inlineStr"/>
+      <c r="U560" s="3" t="inlineStr"/>
+      <c r="V560" s="3" t="inlineStr"/>
+      <c r="W560" s="3" t="inlineStr"/>
+    </row>
+    <row r="561">
+      <c r="A561" s="3" t="inlineStr">
+        <is>
+          <t>gambling-immoral</t>
+        </is>
+      </c>
+      <c r="B561" s="3" t="inlineStr"/>
+      <c r="C561" s="3" t="inlineStr"/>
+      <c r="D561" s="3" t="inlineStr"/>
+      <c r="E561" s="3" t="inlineStr"/>
+      <c r="F561" s="3" t="inlineStr"/>
+      <c r="G561" s="3" t="inlineStr"/>
+      <c r="H561" s="3" t="inlineStr"/>
+      <c r="I561" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="J561" s="3" t="inlineStr">
+        <is>
+          <t>🇩🇪</t>
+        </is>
+      </c>
+      <c r="K561" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="L561" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M561" s="3" t="inlineStr"/>
+      <c r="N561" s="3" t="inlineStr"/>
+      <c r="O561" s="3" t="inlineStr"/>
+      <c r="P561" s="3" t="inlineStr"/>
+      <c r="Q561" s="3" t="inlineStr"/>
+      <c r="R561" s="3" t="inlineStr"/>
+      <c r="S561" s="3" t="inlineStr"/>
+      <c r="T561" s="3" t="inlineStr"/>
+      <c r="U561" s="3" t="inlineStr"/>
+      <c r="V561" s="3" t="inlineStr"/>
+      <c r="W561" s="3" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" s="3" t="inlineStr">
+        <is>
+          <t>gambling-immoral</t>
+        </is>
+      </c>
+      <c r="B562" s="3" t="inlineStr"/>
+      <c r="C562" s="3" t="inlineStr"/>
+      <c r="D562" s="3" t="inlineStr"/>
+      <c r="E562" s="3" t="inlineStr"/>
+      <c r="F562" s="3" t="inlineStr"/>
+      <c r="G562" s="3" t="inlineStr"/>
+      <c r="H562" s="3" t="inlineStr"/>
+      <c r="I562" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="J562" s="3" t="inlineStr">
+        <is>
+          <t>🇺🇸</t>
+        </is>
+      </c>
+      <c r="K562" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="L562" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M562" s="3" t="inlineStr"/>
+      <c r="N562" s="3" t="inlineStr"/>
+      <c r="O562" s="3" t="inlineStr"/>
+      <c r="P562" s="3" t="inlineStr"/>
+      <c r="Q562" s="3" t="inlineStr"/>
+      <c r="R562" s="3" t="inlineStr"/>
+      <c r="S562" s="3" t="inlineStr"/>
+      <c r="T562" s="3" t="inlineStr"/>
+      <c r="U562" s="3" t="inlineStr"/>
+      <c r="V562" s="3" t="inlineStr"/>
+      <c r="W562" s="3" t="inlineStr"/>
+    </row>
+    <row r="563">
+      <c r="A563" s="2" t="inlineStr">
+        <is>
+          <t>gambling-immoral-b</t>
+        </is>
+      </c>
+      <c r="B563" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="C563" s="2" t="inlineStr">
+        <is>
+          <t>🎲</t>
+        </is>
+      </c>
+      <c r="D563" s="2" t="inlineStr">
+        <is>
+          <t>% who say gambling is morally wrong</t>
+        </is>
+      </c>
+      <c r="E563" s="2" t="inlineStr">
+        <is>
+          <t>Gambling is morally unacceptable (US: morally wrong)</t>
+        </is>
+      </c>
+      <c r="F563" s="2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G563" s="2" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H563" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I563" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="J563" s="2" t="inlineStr">
+        <is>
+          <t>🇮🇳</t>
+        </is>
+      </c>
+      <c r="K563" s="2" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="L563" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M563" s="2" t="inlineStr">
+        <is>
+          <t>Pew Research Center Spring 2025 Global Attitudes (Q17d gambling)</t>
+        </is>
+      </c>
+      <c r="N563" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pewresearch.org/short-reads/2026/03/16/americans-are-less-likely-than-people-in-many-other-countries-to-see-gambling-as-morally-wrong/</t>
+        </is>
+      </c>
+      <c r="O563" s="2" t="inlineStr">
+        <is>
+          <t>India (83%) and South Korea (78%) top this set; Brazil and Kenya tie at 61%. Canadians (27%) are even less likely than Americans to say gambling is morally wrong.</t>
+        </is>
+      </c>
+      <c r="P563" s="2" t="inlineStr"/>
+      <c r="Q563" s="2" t="inlineStr"/>
+      <c r="R563" s="2" t="inlineStr"/>
+      <c r="S563" s="2" t="inlineStr">
+        <is>
+          <t>sparkles</t>
+        </is>
+      </c>
+      <c r="T563" s="2" t="inlineStr"/>
+      <c r="U563" s="2" t="inlineStr">
+        <is>
+          <t>pew-gambling-immoral</t>
+        </is>
+      </c>
+      <c r="V563" s="2" t="inlineStr">
+        <is>
+          <t>Gambling Immoral</t>
+        </is>
+      </c>
+      <c r="W563" s="2" t="inlineStr">
+        <is>
+          <t>Snake Eyes</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="inlineStr">
+        <is>
+          <t>gambling-immoral-b</t>
+        </is>
+      </c>
+      <c r="B564" s="2" t="inlineStr"/>
+      <c r="C564" s="2" t="inlineStr"/>
+      <c r="D564" s="2" t="inlineStr"/>
+      <c r="E564" s="2" t="inlineStr"/>
+      <c r="F564" s="2" t="inlineStr"/>
+      <c r="G564" s="2" t="inlineStr"/>
+      <c r="H564" s="2" t="inlineStr"/>
+      <c r="I564" s="2" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="J564" s="2" t="inlineStr">
+        <is>
+          <t>🇰🇷</t>
+        </is>
+      </c>
+      <c r="K564" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="L564" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M564" s="2" t="inlineStr"/>
+      <c r="N564" s="2" t="inlineStr"/>
+      <c r="O564" s="2" t="inlineStr"/>
+      <c r="P564" s="2" t="inlineStr"/>
+      <c r="Q564" s="2" t="inlineStr"/>
+      <c r="R564" s="2" t="inlineStr"/>
+      <c r="S564" s="2" t="inlineStr"/>
+      <c r="T564" s="2" t="inlineStr"/>
+      <c r="U564" s="2" t="inlineStr"/>
+      <c r="V564" s="2" t="inlineStr"/>
+      <c r="W564" s="2" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" s="2" t="inlineStr">
+        <is>
+          <t>gambling-immoral-b</t>
+        </is>
+      </c>
+      <c r="B565" s="2" t="inlineStr"/>
+      <c r="C565" s="2" t="inlineStr"/>
+      <c r="D565" s="2" t="inlineStr"/>
+      <c r="E565" s="2" t="inlineStr"/>
+      <c r="F565" s="2" t="inlineStr"/>
+      <c r="G565" s="2" t="inlineStr"/>
+      <c r="H565" s="2" t="inlineStr"/>
+      <c r="I565" s="2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="J565" s="2" t="inlineStr">
+        <is>
+          <t>🇧🇷</t>
+        </is>
+      </c>
+      <c r="K565" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="L565" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M565" s="2" t="inlineStr"/>
+      <c r="N565" s="2" t="inlineStr"/>
+      <c r="O565" s="2" t="inlineStr"/>
+      <c r="P565" s="2" t="inlineStr"/>
+      <c r="Q565" s="2" t="inlineStr"/>
+      <c r="R565" s="2" t="inlineStr"/>
+      <c r="S565" s="2" t="inlineStr"/>
+      <c r="T565" s="2" t="inlineStr"/>
+      <c r="U565" s="2" t="inlineStr"/>
+      <c r="V565" s="2" t="inlineStr"/>
+      <c r="W565" s="2" t="inlineStr"/>
+    </row>
+    <row r="566">
+      <c r="A566" s="2" t="inlineStr">
+        <is>
+          <t>gambling-immoral-b</t>
+        </is>
+      </c>
+      <c r="B566" s="2" t="inlineStr"/>
+      <c r="C566" s="2" t="inlineStr"/>
+      <c r="D566" s="2" t="inlineStr"/>
+      <c r="E566" s="2" t="inlineStr"/>
+      <c r="F566" s="2" t="inlineStr"/>
+      <c r="G566" s="2" t="inlineStr"/>
+      <c r="H566" s="2" t="inlineStr"/>
+      <c r="I566" s="2" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="J566" s="2" t="inlineStr">
+        <is>
+          <t>🇰🇪</t>
+        </is>
+      </c>
+      <c r="K566" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="L566" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M566" s="2" t="inlineStr"/>
+      <c r="N566" s="2" t="inlineStr"/>
+      <c r="O566" s="2" t="inlineStr"/>
+      <c r="P566" s="2" t="inlineStr"/>
+      <c r="Q566" s="2" t="inlineStr"/>
+      <c r="R566" s="2" t="inlineStr"/>
+      <c r="S566" s="2" t="inlineStr"/>
+      <c r="T566" s="2" t="inlineStr"/>
+      <c r="U566" s="2" t="inlineStr"/>
+      <c r="V566" s="2" t="inlineStr"/>
+      <c r="W566" s="2" t="inlineStr"/>
+    </row>
+    <row r="567">
+      <c r="A567" s="2" t="inlineStr">
+        <is>
+          <t>gambling-immoral-b</t>
+        </is>
+      </c>
+      <c r="B567" s="2" t="inlineStr"/>
+      <c r="C567" s="2" t="inlineStr"/>
+      <c r="D567" s="2" t="inlineStr"/>
+      <c r="E567" s="2" t="inlineStr"/>
+      <c r="F567" s="2" t="inlineStr"/>
+      <c r="G567" s="2" t="inlineStr"/>
+      <c r="H567" s="2" t="inlineStr"/>
+      <c r="I567" s="2" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="J567" s="2" t="inlineStr">
+        <is>
+          <t>🇵🇱</t>
+        </is>
+      </c>
+      <c r="K567" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="L567" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M567" s="2" t="inlineStr"/>
+      <c r="N567" s="2" t="inlineStr"/>
+      <c r="O567" s="2" t="inlineStr"/>
+      <c r="P567" s="2" t="inlineStr"/>
+      <c r="Q567" s="2" t="inlineStr"/>
+      <c r="R567" s="2" t="inlineStr"/>
+      <c r="S567" s="2" t="inlineStr"/>
+      <c r="T567" s="2" t="inlineStr"/>
+      <c r="U567" s="2" t="inlineStr"/>
+      <c r="V567" s="2" t="inlineStr"/>
+      <c r="W567" s="2" t="inlineStr"/>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="inlineStr">
+        <is>
+          <t>gambling-immoral-b</t>
+        </is>
+      </c>
+      <c r="B568" s="2" t="inlineStr"/>
+      <c r="C568" s="2" t="inlineStr"/>
+      <c r="D568" s="2" t="inlineStr"/>
+      <c r="E568" s="2" t="inlineStr"/>
+      <c r="F568" s="2" t="inlineStr"/>
+      <c r="G568" s="2" t="inlineStr"/>
+      <c r="H568" s="2" t="inlineStr"/>
+      <c r="I568" s="2" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="J568" s="2" t="inlineStr">
+        <is>
+          <t>🇨🇦</t>
+        </is>
+      </c>
+      <c r="K568" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="L568" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="M568" s="2" t="inlineStr"/>
+      <c r="N568" s="2" t="inlineStr"/>
+      <c r="O568" s="2" t="inlineStr"/>
+      <c r="P568" s="2" t="inlineStr"/>
+      <c r="Q568" s="2" t="inlineStr"/>
+      <c r="R568" s="2" t="inlineStr"/>
+      <c r="S568" s="2" t="inlineStr"/>
+      <c r="T568" s="2" t="inlineStr"/>
+      <c r="U568" s="2" t="inlineStr"/>
+      <c r="V568" s="2" t="inlineStr"/>
+      <c r="W568" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W556"/>
+  <autoFilter ref="A1:W568"/>
   <dataValidations count="2">
     <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"top,bottom"</formula1>
@@ -82456,7 +83106,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -82669,7 +83319,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -82740,7 +83390,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -82816,7 +83466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -83178,7 +83828,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -83483,7 +84133,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -83851,7 +84501,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
@@ -84141,13 +84791,803 @@
       <c r="P21" s="3" t="inlineStr"/>
       <c r="Q21" s="3" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>match-pew-meaning</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>💭</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>What Matters Most</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Where people found meaning in life (Pew 2021)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>GBR</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>🇬🇧</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>This country mentioned hobbies more than any other surveyed</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Around one-in-five (22%) in the UK mentioned hobbies — the highest share of the 17 publics, and the third most-cited source there after family and friends.</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Pew Research Center: What Makes Life Meaningful? (Spring 2021 Global Attitudes)</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pewresearch.org/global/2021/11/18/what-makes-life-meaningful-views-from-17-advanced-economies/</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>heart</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>match-pew-meaning</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>KOR</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>🇰🇷</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>This country ranked material well-being as its top source of meaning</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>In South Korea, material well-being emerged as the top source of meaning (ahead of health and family), even though fewer people mention multiple topics than in many other publics.</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Pew Research Center: What Makes Life Meaningful? (Spring 2021 Global Attitudes)</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pewresearch.org/global/2021/11/18/what-makes-life-meaningful-views-from-17-advanced-economies/</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>match-pew-meaning</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>TWN</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>🇹🇼</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>This country ranked society as its top source of meaning</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>In Taiwan, society / places / institutions was the top source of meaning (38%), above family, occupation and material well-being — unique among the 17 publics.</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Pew Research Center: What Makes Life Meaningful? (Spring 2021 Global Attitudes)</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pewresearch.org/global/2021/11/18/what-makes-life-meaningful-views-from-17-advanced-economies/</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>match-pew-meaning</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>🇪🇸</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>This country ranked health as its top source of meaning</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>In Spain, 48% mentioned health — the top source of meaning for Spaniards, and the highest health share across the 17 publics.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Pew Research Center: What Makes Life Meaningful? (Spring 2021 Global Attitudes)</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pewresearch.org/global/2021/11/18/what-makes-life-meaningful-views-from-17-advanced-economies/</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>match-pew-meaning</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>🇮🇹</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>This country mentioned occupation more than any other surveyed</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Italy had the highest occupation/career mention rate at 43%, tying family as a top source there; South Korea was lowest at 6%.</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Pew Research Center: What Makes Life Meaningful? (Spring 2021 Global Attitudes)</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pewresearch.org/global/2021/11/18/what-makes-life-meaningful-views-from-17-advanced-economies/</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q21"/>
+  <autoFilter ref="A1:Q26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>puzzle_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>daily_order</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>puzzle_emoji</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>headline</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>subtitle</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>stat_label</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>fun_fact</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>art</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>tier_value</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>tier_label</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>item_name</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>item_emoji</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>country_iso</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>item_value</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>data_year</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>support_url</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>pew-meaning-religion</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>105</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>🙏</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>God is Meaningful</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>% who mentioned religion as a source of meaning in life (Pew 2021)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Spirituality, faith and religion mentioned as a source of meaning</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pew Research Center: What Makes Life Meaningful? Views From 17 Advanced Economies (Spring 2021 Global Attitudes, Q36)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.pewresearch.org/global/2021/11/18/what-makes-life-meaningful-views-from-17-advanced-economies/</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Americans stand out: 15% mentioned religion/God as a source of meaning — three times New Zealand (5%) and far above every other public surveyed (none above 5%).</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>candle</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>🇺🇸</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>pew-meaning-religion</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>pew-meaning-religion</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>🇦🇺</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>AUS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>pew-meaning-religion</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>🇬🇧</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>GBR</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>pew-meaning-religion</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>🇮🇹</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>pew-meaning-religion</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>🇩🇪</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>pew-meaning-religion</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>🇯🇵</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>JPN</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:U7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>